<commit_message>
dados: 2026-10-12 10:19 (106 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/dre/DRE_01_2026.xlsx
+++ b/xlsx/dre/DRE_01_2026.xlsx
@@ -426,6 +426,15 @@
     <t>R$  18.630,00</t>
   </si>
   <si>
+    <t>51101FIN/1</t>
+  </si>
+  <si>
+    <t>R$  7.032,00</t>
+  </si>
+  <si>
+    <t>16/01/26</t>
+  </si>
+  <si>
     <t>56101FIN/1</t>
   </si>
   <si>
@@ -441,13 +450,19 @@
     <t>R$  24.250,23</t>
   </si>
   <si>
-    <t>16/01/26</t>
-  </si>
-  <si>
-    <t>51101FIN/1</t>
-  </si>
-  <si>
-    <t>R$  7.032,00</t>
+    <t>55301FIN/1</t>
+  </si>
+  <si>
+    <t>Gabriella Ferreira da Silva</t>
+  </si>
+  <si>
+    <t>R$  24.000,00</t>
+  </si>
+  <si>
+    <t>26/01/26</t>
+  </si>
+  <si>
+    <t>17/01/26</t>
   </si>
   <si>
     <t>52801FIN/1</t>
@@ -459,21 +474,6 @@
     <t>R$  5.145,00</t>
   </si>
   <si>
-    <t>55301FIN/1</t>
-  </si>
-  <si>
-    <t>Gabriella Ferreira da Silva</t>
-  </si>
-  <si>
-    <t>R$  24.000,00</t>
-  </si>
-  <si>
-    <t>26/01/26</t>
-  </si>
-  <si>
-    <t>17/01/26</t>
-  </si>
-  <si>
     <t>56101/0</t>
   </si>
   <si>
@@ -483,6 +483,15 @@
     <t>56101TadeuTM</t>
   </si>
   <si>
+    <t>58101/0</t>
+  </si>
+  <si>
+    <t>R$  5.000,00</t>
+  </si>
+  <si>
+    <t>58101LucieneBRJ</t>
+  </si>
+  <si>
     <t>53901FIN/1</t>
   </si>
   <si>
@@ -501,15 +510,6 @@
     <t>R$  8.000,00</t>
   </si>
   <si>
-    <t>58101/0</t>
-  </si>
-  <si>
-    <t>R$  5.000,00</t>
-  </si>
-  <si>
-    <t>58101LucieneBRJ</t>
-  </si>
-  <si>
     <t>52201FIN/1</t>
   </si>
   <si>
@@ -750,6 +750,24 @@
     <t>R$  10.440,08</t>
   </si>
   <si>
+    <t>57701/1</t>
+  </si>
+  <si>
+    <t>R$  21.103,49</t>
+  </si>
+  <si>
+    <t>56501/1</t>
+  </si>
+  <si>
+    <t>R$  45,51</t>
+  </si>
+  <si>
+    <t>56101/1</t>
+  </si>
+  <si>
+    <t>R$  7.979,45</t>
+  </si>
+  <si>
     <t>55301/1</t>
   </si>
   <si>
@@ -789,48 +807,39 @@
     <t>R$  8.963,06</t>
   </si>
   <si>
+    <t>58101/1</t>
+  </si>
+  <si>
+    <t>R$  7.830,80</t>
+  </si>
+  <si>
+    <t>56901/1</t>
+  </si>
+  <si>
+    <t>R$  3.822,66</t>
+  </si>
+  <si>
     <t>52601/1</t>
   </si>
   <si>
     <t>R$  4.879,58</t>
   </si>
   <si>
-    <t>57701/1</t>
-  </si>
-  <si>
-    <t>R$  21.103,49</t>
-  </si>
-  <si>
-    <t>58101/1</t>
-  </si>
-  <si>
-    <t>R$  7.830,80</t>
-  </si>
-  <si>
-    <t>56901/1</t>
-  </si>
-  <si>
-    <t>R$  3.822,66</t>
-  </si>
-  <si>
-    <t>56101/1</t>
-  </si>
-  <si>
-    <t>R$  7.979,45</t>
-  </si>
-  <si>
-    <t>56501/1</t>
-  </si>
-  <si>
-    <t>R$  45,51</t>
-  </si>
-  <si>
     <t>58901/1</t>
   </si>
   <si>
     <t>R$  3.866,37</t>
   </si>
   <si>
+    <t>54401/1</t>
+  </si>
+  <si>
+    <t>R$  9.694,52</t>
+  </si>
+  <si>
+    <t>GIR</t>
+  </si>
+  <si>
     <t>53501/1</t>
   </si>
   <si>
@@ -838,45 +847,6 @@
   </si>
   <si>
     <t>53501CassioMMP</t>
-  </si>
-  <si>
-    <t>54401/1</t>
-  </si>
-  <si>
-    <t>R$  9.694,52</t>
-  </si>
-  <si>
-    <t>GIR</t>
-  </si>
-  <si>
-    <t>R$  206,07</t>
-  </si>
-  <si>
-    <t>57201/1</t>
-  </si>
-  <si>
-    <t>R$  478,43</t>
-  </si>
-  <si>
-    <t>23/01/26</t>
-  </si>
-  <si>
-    <t>57201MarinaA</t>
-  </si>
-  <si>
-    <t>R$  585,09</t>
-  </si>
-  <si>
-    <t>56801/1</t>
-  </si>
-  <si>
-    <t>R$  16.857,19</t>
-  </si>
-  <si>
-    <t>GiR</t>
-  </si>
-  <si>
-    <t>56801ArytanaDAST</t>
   </si>
   <si>
     <t>53501/2</t>
@@ -892,16 +862,55 @@
 </t>
   </si>
   <si>
+    <t>R$  206,07</t>
+  </si>
+  <si>
+    <t>57201/1</t>
+  </si>
+  <si>
+    <t>R$  478,43</t>
+  </si>
+  <si>
+    <t>23/01/26</t>
+  </si>
+  <si>
+    <t>57201MarinaA</t>
+  </si>
+  <si>
+    <t>56801/1</t>
+  </si>
+  <si>
+    <t>R$  16.857,19</t>
+  </si>
+  <si>
+    <t>GiR</t>
+  </si>
+  <si>
+    <t>56801ArytanaDAST</t>
+  </si>
+  <si>
+    <t>58201/2</t>
+  </si>
+  <si>
+    <t>R$  15.368,23</t>
+  </si>
+  <si>
+    <t>56801/2</t>
+  </si>
+  <si>
+    <t>R$  460,43</t>
+  </si>
+  <si>
+    <t>R$  585,09</t>
+  </si>
+  <si>
     <t>51101/2</t>
   </si>
   <si>
     <t>R$  155,40</t>
   </si>
   <si>
-    <t>58201/2</t>
-  </si>
-  <si>
-    <t>R$  15.368,23</t>
+    <t>R$  4.159,95</t>
   </si>
   <si>
     <t>58201/3</t>
@@ -910,19 +919,10 @@
     <t>R$  66,29</t>
   </si>
   <si>
-    <t>56801/2</t>
-  </si>
-  <si>
-    <t>R$  460,43</t>
-  </si>
-  <si>
     <t>56801/3</t>
   </si>
   <si>
     <t>R$  1.544,84</t>
-  </si>
-  <si>
-    <t>R$  4.159,95</t>
   </si>
   <si>
     <t>R$  1.856,90</t>
@@ -5035,16 +5035,16 @@
         <v>41</v>
       </c>
       <c r="H44" t="s">
+        <v>110</v>
+      </c>
+      <c r="I44" t="s">
         <v>138</v>
       </c>
-      <c r="I44" t="s">
+      <c r="J44" t="s">
         <v>139</v>
       </c>
-      <c r="J44" t="s">
-        <v>133</v>
-      </c>
       <c r="K44" t="s">
-        <v>134</v>
+        <v>111</v>
       </c>
       <c r="L44" t="s">
         <v>84</v>
@@ -5091,16 +5091,16 @@
         <v>41</v>
       </c>
       <c r="H45" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="I45" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J45" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="K45" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="L45" t="s">
         <v>84</v>
@@ -5147,16 +5147,16 @@
         <v>41</v>
       </c>
       <c r="H46" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="I46" t="s">
         <v>144</v>
       </c>
       <c r="J46" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="K46" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L46" t="s">
         <v>84</v>
@@ -5209,10 +5209,10 @@
         <v>147</v>
       </c>
       <c r="J47" t="s">
-        <v>89</v>
+        <v>148</v>
       </c>
       <c r="K47" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="L47" t="s">
         <v>84</v>
@@ -5250,7 +5250,7 @@
         <v>34</v>
       </c>
       <c r="E48" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F48" t="s">
         <v>80</v>
@@ -5259,16 +5259,16 @@
         <v>41</v>
       </c>
       <c r="H48" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I48" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J48" t="s">
-        <v>151</v>
+        <v>89</v>
       </c>
       <c r="K48" t="s">
-        <v>152</v>
+        <v>133</v>
       </c>
       <c r="L48" t="s">
         <v>84</v>
@@ -5315,7 +5315,7 @@
         <v>41</v>
       </c>
       <c r="H49" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I49" t="s">
         <v>154</v>
@@ -5365,25 +5365,25 @@
         <v>156</v>
       </c>
       <c r="F50" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="G50" t="s">
         <v>41</v>
       </c>
       <c r="H50" t="s">
+        <v>86</v>
+      </c>
+      <c r="I50" t="s">
         <v>157</v>
       </c>
-      <c r="I50" t="s">
-        <v>158</v>
-      </c>
       <c r="J50" t="s">
-        <v>128</v>
+        <v>89</v>
       </c>
       <c r="K50" t="s">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="L50" t="s">
-        <v>84</v>
+        <v>34</v>
       </c>
       <c r="M50" t="s">
         <v>77</v>
@@ -5392,13 +5392,13 @@
         <v>47</v>
       </c>
       <c r="O50" t="s">
-        <v>34</v>
+        <v>158</v>
       </c>
       <c r="P50" t="s">
-        <v>34</v>
+        <v>157</v>
       </c>
       <c r="Q50" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R50" t="s">
         <v>34</v>
@@ -5433,7 +5433,7 @@
         <v>161</v>
       </c>
       <c r="J51" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="K51" t="s">
         <v>111</v>
@@ -5477,25 +5477,25 @@
         <v>162</v>
       </c>
       <c r="F52" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G52" t="s">
         <v>41</v>
       </c>
       <c r="H52" t="s">
-        <v>86</v>
+        <v>163</v>
       </c>
       <c r="I52" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J52" t="s">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="K52" t="s">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="L52" t="s">
-        <v>34</v>
+        <v>84</v>
       </c>
       <c r="M52" t="s">
         <v>77</v>
@@ -5504,13 +5504,13 @@
         <v>47</v>
       </c>
       <c r="O52" t="s">
-        <v>164</v>
+        <v>34</v>
       </c>
       <c r="P52" t="s">
-        <v>163</v>
+        <v>34</v>
       </c>
       <c r="Q52" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R52" t="s">
         <v>34</v>
@@ -6889,10 +6889,10 @@
         <v>246</v>
       </c>
       <c r="J77" t="s">
-        <v>152</v>
+        <v>83</v>
       </c>
       <c r="K77" t="s">
-        <v>152</v>
+        <v>70</v>
       </c>
       <c r="L77" t="s">
         <v>34</v>
@@ -6904,13 +6904,13 @@
         <v>47</v>
       </c>
       <c r="O77" t="s">
-        <v>34</v>
+        <v>173</v>
       </c>
       <c r="P77" t="s">
-        <v>34</v>
+        <v>246</v>
       </c>
       <c r="Q77" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R77" t="s">
         <v>34</v>
@@ -6945,10 +6945,10 @@
         <v>248</v>
       </c>
       <c r="J78" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="K78" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="L78" t="s">
         <v>34</v>
@@ -6960,13 +6960,13 @@
         <v>47</v>
       </c>
       <c r="O78" t="s">
-        <v>112</v>
+        <v>34</v>
       </c>
       <c r="P78" t="s">
-        <v>248</v>
+        <v>34</v>
       </c>
       <c r="Q78" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R78" t="s">
         <v>34</v>
@@ -7001,10 +7001,10 @@
         <v>250</v>
       </c>
       <c r="J79" t="s">
-        <v>97</v>
+        <v>134</v>
       </c>
       <c r="K79" t="s">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="L79" t="s">
         <v>34</v>
@@ -7016,7 +7016,7 @@
         <v>47</v>
       </c>
       <c r="O79" t="s">
-        <v>98</v>
+        <v>155</v>
       </c>
       <c r="P79" t="s">
         <v>250</v>
@@ -7057,10 +7057,10 @@
         <v>252</v>
       </c>
       <c r="J80" t="s">
-        <v>58</v>
+        <v>149</v>
       </c>
       <c r="K80" t="s">
-        <v>58</v>
+        <v>149</v>
       </c>
       <c r="L80" t="s">
         <v>34</v>
@@ -7072,13 +7072,13 @@
         <v>47</v>
       </c>
       <c r="O80" t="s">
-        <v>253</v>
+        <v>34</v>
       </c>
       <c r="P80" t="s">
-        <v>252</v>
+        <v>34</v>
       </c>
       <c r="Q80" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R80" t="s">
         <v>34</v>
@@ -7098,7 +7098,7 @@
         <v>34</v>
       </c>
       <c r="E81" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F81" t="s">
         <v>242</v>
@@ -7110,7 +7110,7 @@
         <v>243</v>
       </c>
       <c r="I81" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="J81" t="s">
         <v>111</v>
@@ -7128,13 +7128,13 @@
         <v>47</v>
       </c>
       <c r="O81" t="s">
-        <v>34</v>
+        <v>112</v>
       </c>
       <c r="P81" t="s">
-        <v>34</v>
+        <v>254</v>
       </c>
       <c r="Q81" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R81" t="s">
         <v>34</v>
@@ -7154,7 +7154,7 @@
         <v>34</v>
       </c>
       <c r="E82" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F82" t="s">
         <v>242</v>
@@ -7166,13 +7166,13 @@
         <v>243</v>
       </c>
       <c r="I82" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J82" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="K82" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="L82" t="s">
         <v>34</v>
@@ -7184,13 +7184,13 @@
         <v>47</v>
       </c>
       <c r="O82" t="s">
-        <v>34</v>
+        <v>98</v>
       </c>
       <c r="P82" t="s">
-        <v>34</v>
+        <v>256</v>
       </c>
       <c r="Q82" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R82" t="s">
         <v>34</v>
@@ -7210,7 +7210,7 @@
         <v>34</v>
       </c>
       <c r="E83" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F83" t="s">
         <v>242</v>
@@ -7222,13 +7222,13 @@
         <v>243</v>
       </c>
       <c r="I83" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="J83" t="s">
-        <v>107</v>
+        <v>58</v>
       </c>
       <c r="K83" t="s">
-        <v>107</v>
+        <v>58</v>
       </c>
       <c r="L83" t="s">
         <v>34</v>
@@ -7240,13 +7240,13 @@
         <v>47</v>
       </c>
       <c r="O83" t="s">
-        <v>34</v>
+        <v>259</v>
       </c>
       <c r="P83" t="s">
-        <v>34</v>
+        <v>258</v>
       </c>
       <c r="Q83" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R83" t="s">
         <v>34</v>
@@ -7281,10 +7281,10 @@
         <v>261</v>
       </c>
       <c r="J84" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="K84" t="s">
-        <v>70</v>
+        <v>111</v>
       </c>
       <c r="L84" t="s">
         <v>34</v>
@@ -7296,13 +7296,13 @@
         <v>47</v>
       </c>
       <c r="O84" t="s">
-        <v>173</v>
+        <v>34</v>
       </c>
       <c r="P84" t="s">
-        <v>261</v>
+        <v>34</v>
       </c>
       <c r="Q84" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R84" t="s">
         <v>34</v>
@@ -7393,10 +7393,10 @@
         <v>265</v>
       </c>
       <c r="J86" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="K86" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="L86" t="s">
         <v>34</v>
@@ -7449,7 +7449,7 @@
         <v>267</v>
       </c>
       <c r="J87" t="s">
-        <v>134</v>
+        <v>70</v>
       </c>
       <c r="K87" t="s">
         <v>70</v>
@@ -7464,13 +7464,13 @@
         <v>47</v>
       </c>
       <c r="O87" t="s">
-        <v>155</v>
+        <v>34</v>
       </c>
       <c r="P87" t="s">
-        <v>267</v>
+        <v>34</v>
       </c>
       <c r="Q87" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R87" t="s">
         <v>34</v>
@@ -7505,10 +7505,10 @@
         <v>269</v>
       </c>
       <c r="J88" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="K88" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="L88" t="s">
         <v>34</v>
@@ -7617,13 +7617,13 @@
         <v>273</v>
       </c>
       <c r="J90" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="K90" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L90" t="s">
-        <v>34</v>
+        <v>274</v>
       </c>
       <c r="M90" t="s">
         <v>236</v>
@@ -7632,7 +7632,7 @@
         <v>47</v>
       </c>
       <c r="O90" t="s">
-        <v>274</v>
+        <v>120</v>
       </c>
       <c r="P90" t="s">
         <v>273</v>
@@ -7673,13 +7673,13 @@
         <v>276</v>
       </c>
       <c r="J91" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="K91" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L91" t="s">
-        <v>277</v>
+        <v>34</v>
       </c>
       <c r="M91" t="s">
         <v>236</v>
@@ -7688,7 +7688,7 @@
         <v>47</v>
       </c>
       <c r="O91" t="s">
-        <v>120</v>
+        <v>277</v>
       </c>
       <c r="P91" t="s">
         <v>276</v>
@@ -7714,7 +7714,7 @@
         <v>34</v>
       </c>
       <c r="E92" t="s">
-        <v>249</v>
+        <v>278</v>
       </c>
       <c r="F92" t="s">
         <v>212</v>
@@ -7723,19 +7723,19 @@
         <v>41</v>
       </c>
       <c r="H92" t="s">
-        <v>243</v>
+        <v>279</v>
       </c>
       <c r="I92" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="J92" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="K92" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="L92" t="s">
-        <v>34</v>
+        <v>281</v>
       </c>
       <c r="M92" t="s">
         <v>236</v>
@@ -7744,10 +7744,10 @@
         <v>47</v>
       </c>
       <c r="O92" t="s">
-        <v>98</v>
+        <v>277</v>
       </c>
       <c r="P92" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="Q92" t="s">
         <v>47</v>
@@ -7770,7 +7770,7 @@
         <v>34</v>
       </c>
       <c r="E93" t="s">
-        <v>279</v>
+        <v>255</v>
       </c>
       <c r="F93" t="s">
         <v>212</v>
@@ -7782,13 +7782,13 @@
         <v>243</v>
       </c>
       <c r="I93" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="J93" t="s">
-        <v>281</v>
+        <v>97</v>
       </c>
       <c r="K93" t="s">
-        <v>281</v>
+        <v>97</v>
       </c>
       <c r="L93" t="s">
         <v>34</v>
@@ -7800,10 +7800,10 @@
         <v>47</v>
       </c>
       <c r="O93" t="s">
+        <v>98</v>
+      </c>
+      <c r="P93" t="s">
         <v>282</v>
-      </c>
-      <c r="P93" t="s">
-        <v>280</v>
       </c>
       <c r="Q93" t="s">
         <v>47</v>
@@ -7826,7 +7826,7 @@
         <v>34</v>
       </c>
       <c r="E94" t="s">
-        <v>241</v>
+        <v>283</v>
       </c>
       <c r="F94" t="s">
         <v>212</v>
@@ -7838,13 +7838,13 @@
         <v>243</v>
       </c>
       <c r="I94" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="J94" t="s">
-        <v>128</v>
+        <v>285</v>
       </c>
       <c r="K94" t="s">
-        <v>102</v>
+        <v>285</v>
       </c>
       <c r="L94" t="s">
         <v>34</v>
@@ -7856,10 +7856,10 @@
         <v>47</v>
       </c>
       <c r="O94" t="s">
-        <v>103</v>
+        <v>286</v>
       </c>
       <c r="P94" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="Q94" t="s">
         <v>47</v>
@@ -7882,7 +7882,7 @@
         <v>34</v>
       </c>
       <c r="E95" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F95" t="s">
         <v>212</v>
@@ -7894,7 +7894,7 @@
         <v>243</v>
       </c>
       <c r="I95" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="J95" t="s">
         <v>83</v>
@@ -7903,7 +7903,7 @@
         <v>119</v>
       </c>
       <c r="L95" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="M95" t="s">
         <v>236</v>
@@ -7912,10 +7912,10 @@
         <v>47</v>
       </c>
       <c r="O95" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P95" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="Q95" t="s">
         <v>47</v>
@@ -7938,7 +7938,7 @@
         <v>34</v>
       </c>
       <c r="E96" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="F96" t="s">
         <v>212</v>
@@ -7947,19 +7947,19 @@
         <v>41</v>
       </c>
       <c r="H96" t="s">
-        <v>289</v>
+        <v>243</v>
       </c>
       <c r="I96" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="J96" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="K96" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="L96" t="s">
-        <v>291</v>
+        <v>34</v>
       </c>
       <c r="M96" t="s">
         <v>236</v>
@@ -7968,10 +7968,10 @@
         <v>47</v>
       </c>
       <c r="O96" t="s">
-        <v>274</v>
+        <v>214</v>
       </c>
       <c r="P96" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="Q96" t="s">
         <v>47</v>
@@ -7994,7 +7994,7 @@
         <v>34</v>
       </c>
       <c r="E97" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F97" t="s">
         <v>212</v>
@@ -8006,13 +8006,13 @@
         <v>243</v>
       </c>
       <c r="I97" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J97" t="s">
-        <v>111</v>
+        <v>83</v>
       </c>
       <c r="K97" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L97" t="s">
         <v>34</v>
@@ -8024,10 +8024,10 @@
         <v>47</v>
       </c>
       <c r="O97" t="s">
-        <v>112</v>
+        <v>290</v>
       </c>
       <c r="P97" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="Q97" t="s">
         <v>47</v>
@@ -8050,7 +8050,7 @@
         <v>34</v>
       </c>
       <c r="E98" t="s">
-        <v>294</v>
+        <v>241</v>
       </c>
       <c r="F98" t="s">
         <v>212</v>
@@ -8065,10 +8065,10 @@
         <v>295</v>
       </c>
       <c r="J98" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="K98" t="s">
-        <v>133</v>
+        <v>102</v>
       </c>
       <c r="L98" t="s">
         <v>34</v>
@@ -8080,7 +8080,7 @@
         <v>47</v>
       </c>
       <c r="O98" t="s">
-        <v>214</v>
+        <v>103</v>
       </c>
       <c r="P98" t="s">
         <v>295</v>
@@ -8121,10 +8121,10 @@
         <v>297</v>
       </c>
       <c r="J99" t="s">
-        <v>133</v>
+        <v>111</v>
       </c>
       <c r="K99" t="s">
-        <v>133</v>
+        <v>111</v>
       </c>
       <c r="L99" t="s">
         <v>34</v>
@@ -8136,7 +8136,7 @@
         <v>47</v>
       </c>
       <c r="O99" t="s">
-        <v>214</v>
+        <v>112</v>
       </c>
       <c r="P99" t="s">
         <v>297</v>
@@ -8162,7 +8162,7 @@
         <v>34</v>
       </c>
       <c r="E100" t="s">
-        <v>298</v>
+        <v>287</v>
       </c>
       <c r="F100" t="s">
         <v>212</v>
@@ -8171,10 +8171,10 @@
         <v>41</v>
       </c>
       <c r="H100" t="s">
-        <v>243</v>
+        <v>279</v>
       </c>
       <c r="I100" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J100" t="s">
         <v>83</v>
@@ -8192,10 +8192,10 @@
         <v>47</v>
       </c>
       <c r="O100" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P100" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="Q100" t="s">
         <v>47</v>
@@ -8218,7 +8218,7 @@
         <v>34</v>
       </c>
       <c r="E101" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F101" t="s">
         <v>212</v>
@@ -8230,13 +8230,13 @@
         <v>243</v>
       </c>
       <c r="I101" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J101" t="s">
-        <v>83</v>
+        <v>133</v>
       </c>
       <c r="K101" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="L101" t="s">
         <v>34</v>
@@ -8248,10 +8248,10 @@
         <v>47</v>
       </c>
       <c r="O101" t="s">
-        <v>287</v>
+        <v>214</v>
       </c>
       <c r="P101" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="Q101" t="s">
         <v>47</v>
@@ -8274,7 +8274,7 @@
         <v>34</v>
       </c>
       <c r="E102" t="s">
-        <v>284</v>
+        <v>301</v>
       </c>
       <c r="F102" t="s">
         <v>212</v>
@@ -8283,7 +8283,7 @@
         <v>41</v>
       </c>
       <c r="H102" t="s">
-        <v>289</v>
+        <v>243</v>
       </c>
       <c r="I102" t="s">
         <v>302</v>
@@ -8304,7 +8304,7 @@
         <v>47</v>
       </c>
       <c r="O102" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P102" t="s">
         <v>302</v>
@@ -8330,7 +8330,7 @@
         <v>34</v>
       </c>
       <c r="E103" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="F103" t="s">
         <v>212</v>
@@ -8395,7 +8395,7 @@
         <v>41</v>
       </c>
       <c r="H104" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="I104" t="s">
         <v>304</v>
@@ -8451,7 +8451,7 @@
         <v>41</v>
       </c>
       <c r="H105" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="I105" t="s">
         <v>306</v>
@@ -8472,7 +8472,7 @@
         <v>47</v>
       </c>
       <c r="O105" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P105" t="s">
         <v>306</v>
@@ -10096,7 +10096,7 @@
         <v>47</v>
       </c>
       <c r="O134" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="P134" t="s">
         <v>385</v>
@@ -10137,10 +10137,10 @@
         <v>387</v>
       </c>
       <c r="J135" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="K135" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="L135" t="s">
         <v>361</v>
@@ -10152,7 +10152,7 @@
         <v>47</v>
       </c>
       <c r="O135" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="P135" t="s">
         <v>387</v>
@@ -10178,7 +10178,7 @@
         <v>34</v>
       </c>
       <c r="E136" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="F136" t="s">
         <v>242</v>
@@ -10208,7 +10208,7 @@
         <v>47</v>
       </c>
       <c r="O136" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="P136" t="s">
         <v>385</v>
@@ -10305,10 +10305,10 @@
         <v>390</v>
       </c>
       <c r="J138" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="K138" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="L138" t="s">
         <v>361</v>
@@ -10320,7 +10320,7 @@
         <v>47</v>
       </c>
       <c r="O138" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="P138" t="s">
         <v>390</v>
@@ -10417,10 +10417,10 @@
         <v>394</v>
       </c>
       <c r="J140" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="K140" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L140" t="s">
         <v>361</v>
@@ -10529,10 +10529,10 @@
         <v>399</v>
       </c>
       <c r="J142" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="K142" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L142" t="s">
         <v>361</v>
@@ -10600,7 +10600,7 @@
         <v>47</v>
       </c>
       <c r="O143" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="P143" t="s">
         <v>401</v>
@@ -10656,7 +10656,7 @@
         <v>47</v>
       </c>
       <c r="O144" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="P144" t="s">
         <v>403</v>
@@ -10794,7 +10794,7 @@
         <v>34</v>
       </c>
       <c r="E147" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F147" t="s">
         <v>242</v>
@@ -10824,7 +10824,7 @@
         <v>47</v>
       </c>
       <c r="O147" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P147" t="s">
         <v>408</v>
@@ -10906,7 +10906,7 @@
         <v>34</v>
       </c>
       <c r="E149" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="F149" t="s">
         <v>242</v>
@@ -10962,7 +10962,7 @@
         <v>34</v>
       </c>
       <c r="E150" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="F150" t="s">
         <v>242</v>
@@ -11074,7 +11074,7 @@
         <v>34</v>
       </c>
       <c r="E152" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="F152" t="s">
         <v>242</v>
@@ -11104,7 +11104,7 @@
         <v>47</v>
       </c>
       <c r="O152" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P152" t="s">
         <v>415</v>
@@ -11130,7 +11130,7 @@
         <v>34</v>
       </c>
       <c r="E153" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="F153" t="s">
         <v>242</v>
@@ -11888,7 +11888,7 @@
         <v>47</v>
       </c>
       <c r="O166" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P166" t="s">
         <v>443</v>
@@ -11932,7 +11932,7 @@
         <v>442</v>
       </c>
       <c r="K167" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L167" t="s">
         <v>34</v>
@@ -12041,10 +12041,10 @@
         <v>450</v>
       </c>
       <c r="J169" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="K169" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L169" t="s">
         <v>34</v>
@@ -12168,7 +12168,7 @@
         <v>47</v>
       </c>
       <c r="O171" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P171" t="s">
         <v>453</v>
@@ -12209,10 +12209,10 @@
         <v>454</v>
       </c>
       <c r="J172" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="K172" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L172" t="s">
         <v>34</v>
@@ -12380,7 +12380,7 @@
         <v>442</v>
       </c>
       <c r="K175" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L175" t="s">
         <v>34</v>
@@ -12616,7 +12616,7 @@
         <v>47</v>
       </c>
       <c r="O179" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P179" t="s">
         <v>464</v>
@@ -12840,7 +12840,7 @@
         <v>47</v>
       </c>
       <c r="O183" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P183" t="s">
         <v>470</v>
@@ -13426,7 +13426,7 @@
         <v>33</v>
       </c>
       <c r="E194" t="s">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="F194" t="s">
         <v>242</v>
@@ -13538,7 +13538,7 @@
         <v>34</v>
       </c>
       <c r="E196" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="F196" t="s">
         <v>242</v>
@@ -13650,7 +13650,7 @@
         <v>34</v>
       </c>
       <c r="E198" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="F198" t="s">
         <v>242</v>
@@ -13706,7 +13706,7 @@
         <v>34</v>
       </c>
       <c r="E199" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="F199" t="s">
         <v>242</v>
@@ -13762,7 +13762,7 @@
         <v>34</v>
       </c>
       <c r="E200" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="F200" t="s">
         <v>242</v>
@@ -13874,7 +13874,7 @@
         <v>34</v>
       </c>
       <c r="E202" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F202" t="s">
         <v>242</v>
@@ -13904,7 +13904,7 @@
         <v>47</v>
       </c>
       <c r="O202" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="P202" t="s">
         <v>496</v>
@@ -13930,7 +13930,7 @@
         <v>34</v>
       </c>
       <c r="E203" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="F203" t="s">
         <v>242</v>
@@ -13986,7 +13986,7 @@
         <v>34</v>
       </c>
       <c r="E204" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F204" t="s">
         <v>242</v>
@@ -14004,7 +14004,7 @@
         <v>189</v>
       </c>
       <c r="K204" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L204" t="s">
         <v>34</v>
@@ -14042,7 +14042,7 @@
         <v>34</v>
       </c>
       <c r="E205" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="F205" t="s">
         <v>242</v>
@@ -14098,7 +14098,7 @@
         <v>34</v>
       </c>
       <c r="E206" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="F206" t="s">
         <v>242</v>
@@ -14128,7 +14128,7 @@
         <v>47</v>
       </c>
       <c r="O206" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="P206" t="s">
         <v>502</v>
@@ -14154,7 +14154,7 @@
         <v>34</v>
       </c>
       <c r="E207" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="F207" t="s">
         <v>242</v>
@@ -14184,7 +14184,7 @@
         <v>47</v>
       </c>
       <c r="O207" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="P207" t="s">
         <v>503</v>
@@ -14210,7 +14210,7 @@
         <v>34</v>
       </c>
       <c r="E208" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="F208" t="s">
         <v>242</v>
@@ -14322,7 +14322,7 @@
         <v>34</v>
       </c>
       <c r="E210" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="F210" t="s">
         <v>242</v>
@@ -14378,7 +14378,7 @@
         <v>34</v>
       </c>
       <c r="E211" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F211" t="s">
         <v>242</v>
@@ -14408,7 +14408,7 @@
         <v>47</v>
       </c>
       <c r="O211" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P211" t="s">
         <v>509</v>
@@ -14490,7 +14490,7 @@
         <v>33</v>
       </c>
       <c r="E213" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="F213" t="s">
         <v>242</v>
@@ -14546,7 +14546,7 @@
         <v>34</v>
       </c>
       <c r="E214" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="F214" t="s">
         <v>242</v>
@@ -14658,7 +14658,7 @@
         <v>34</v>
       </c>
       <c r="E216" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F216" t="s">
         <v>242</v>
@@ -14688,7 +14688,7 @@
         <v>47</v>
       </c>
       <c r="O216" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="P216" t="s">
         <v>518</v>
@@ -14714,7 +14714,7 @@
         <v>34</v>
       </c>
       <c r="E217" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="F217" t="s">
         <v>242</v>
@@ -14770,7 +14770,7 @@
         <v>34</v>
       </c>
       <c r="E218" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="F218" t="s">
         <v>242</v>
@@ -14800,7 +14800,7 @@
         <v>47</v>
       </c>
       <c r="O218" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="P218" t="s">
         <v>520</v>
@@ -14826,7 +14826,7 @@
         <v>34</v>
       </c>
       <c r="E219" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="F219" t="s">
         <v>242</v>
@@ -14856,7 +14856,7 @@
         <v>47</v>
       </c>
       <c r="O219" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="P219" t="s">
         <v>522</v>
@@ -14882,7 +14882,7 @@
         <v>34</v>
       </c>
       <c r="E220" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="F220" t="s">
         <v>242</v>
@@ -14912,7 +14912,7 @@
         <v>47</v>
       </c>
       <c r="O220" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="P220" t="s">
         <v>525</v>
@@ -14938,7 +14938,7 @@
         <v>34</v>
       </c>
       <c r="E221" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="F221" t="s">
         <v>242</v>
@@ -14968,7 +14968,7 @@
         <v>47</v>
       </c>
       <c r="O221" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="P221" t="s">
         <v>527</v>
@@ -15050,7 +15050,7 @@
         <v>34</v>
       </c>
       <c r="E223" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F223" t="s">
         <v>242</v>
@@ -15080,7 +15080,7 @@
         <v>47</v>
       </c>
       <c r="O223" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P223" t="s">
         <v>529</v>
@@ -15106,7 +15106,7 @@
         <v>34</v>
       </c>
       <c r="E224" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="F224" t="s">
         <v>242</v>
@@ -15218,7 +15218,7 @@
         <v>34</v>
       </c>
       <c r="E226" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="F226" t="s">
         <v>242</v>
@@ -15274,7 +15274,7 @@
         <v>34</v>
       </c>
       <c r="E227" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F227" t="s">
         <v>242</v>
@@ -15304,7 +15304,7 @@
         <v>47</v>
       </c>
       <c r="O227" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P227" t="s">
         <v>533</v>
@@ -15386,7 +15386,7 @@
         <v>34</v>
       </c>
       <c r="E229" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="F229" t="s">
         <v>242</v>
@@ -15498,7 +15498,7 @@
         <v>34</v>
       </c>
       <c r="E231" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="F231" t="s">
         <v>242</v>
@@ -15554,7 +15554,7 @@
         <v>34</v>
       </c>
       <c r="E232" t="s">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="F232" t="s">
         <v>242</v>
@@ -15610,7 +15610,7 @@
         <v>34</v>
       </c>
       <c r="E233" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="F233" t="s">
         <v>242</v>
@@ -15666,7 +15666,7 @@
         <v>34</v>
       </c>
       <c r="E234" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F234" t="s">
         <v>242</v>
@@ -15684,7 +15684,7 @@
         <v>189</v>
       </c>
       <c r="K234" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L234" t="s">
         <v>34</v>
@@ -15778,7 +15778,7 @@
         <v>34</v>
       </c>
       <c r="E236" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="F236" t="s">
         <v>242</v>
@@ -15890,7 +15890,7 @@
         <v>34</v>
       </c>
       <c r="E238" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="F238" t="s">
         <v>242</v>
@@ -15946,7 +15946,7 @@
         <v>34</v>
       </c>
       <c r="E239" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F239" t="s">
         <v>242</v>
@@ -15964,7 +15964,7 @@
         <v>341</v>
       </c>
       <c r="K239" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L239" t="s">
         <v>34</v>
@@ -16002,7 +16002,7 @@
         <v>34</v>
       </c>
       <c r="E240" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="F240" t="s">
         <v>242</v>
@@ -16058,7 +16058,7 @@
         <v>34</v>
       </c>
       <c r="E241" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="F241" t="s">
         <v>242</v>
@@ -16114,7 +16114,7 @@
         <v>34</v>
       </c>
       <c r="E242" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="F242" t="s">
         <v>242</v>
@@ -16144,7 +16144,7 @@
         <v>47</v>
       </c>
       <c r="O242" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="P242" t="s">
         <v>549</v>
@@ -16170,7 +16170,7 @@
         <v>34</v>
       </c>
       <c r="E243" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F243" t="s">
         <v>242</v>
@@ -16200,7 +16200,7 @@
         <v>47</v>
       </c>
       <c r="O243" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="P243" t="s">
         <v>550</v>
@@ -16226,7 +16226,7 @@
         <v>34</v>
       </c>
       <c r="E244" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="F244" t="s">
         <v>242</v>
@@ -16282,7 +16282,7 @@
         <v>34</v>
       </c>
       <c r="E245" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="F245" t="s">
         <v>242</v>
@@ -16338,7 +16338,7 @@
         <v>34</v>
       </c>
       <c r="E246" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="F246" t="s">
         <v>242</v>
@@ -16368,7 +16368,7 @@
         <v>47</v>
       </c>
       <c r="O246" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="P246" t="s">
         <v>553</v>
@@ -16394,7 +16394,7 @@
         <v>34</v>
       </c>
       <c r="E247" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="F247" t="s">
         <v>242</v>
@@ -16450,7 +16450,7 @@
         <v>34</v>
       </c>
       <c r="E248" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F248" t="s">
         <v>242</v>
@@ -16480,7 +16480,7 @@
         <v>47</v>
       </c>
       <c r="O248" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P248" t="s">
         <v>509</v>
@@ -16506,7 +16506,7 @@
         <v>34</v>
       </c>
       <c r="E249" t="s">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="F249" t="s">
         <v>242</v>
@@ -16562,7 +16562,7 @@
         <v>34</v>
       </c>
       <c r="E250" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="F250" t="s">
         <v>242</v>
@@ -16618,7 +16618,7 @@
         <v>34</v>
       </c>
       <c r="E251" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="F251" t="s">
         <v>242</v>
@@ -16674,7 +16674,7 @@
         <v>34</v>
       </c>
       <c r="E252" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="F252" t="s">
         <v>242</v>
@@ -16704,7 +16704,7 @@
         <v>47</v>
       </c>
       <c r="O252" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="P252" t="s">
         <v>503</v>
@@ -16730,7 +16730,7 @@
         <v>34</v>
       </c>
       <c r="E253" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="F253" t="s">
         <v>242</v>
@@ -16760,7 +16760,7 @@
         <v>47</v>
       </c>
       <c r="O253" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="P253" t="s">
         <v>502</v>
@@ -16786,7 +16786,7 @@
         <v>34</v>
       </c>
       <c r="E254" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="F254" t="s">
         <v>242</v>
@@ -16842,7 +16842,7 @@
         <v>34</v>
       </c>
       <c r="E255" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="F255" t="s">
         <v>242</v>
@@ -16898,7 +16898,7 @@
         <v>34</v>
       </c>
       <c r="E256" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="F256" t="s">
         <v>242</v>
@@ -16954,7 +16954,7 @@
         <v>34</v>
       </c>
       <c r="E257" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="F257" t="s">
         <v>242</v>
@@ -17010,7 +17010,7 @@
         <v>34</v>
       </c>
       <c r="E258" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F258" t="s">
         <v>242</v>
@@ -17028,7 +17028,7 @@
         <v>189</v>
       </c>
       <c r="K258" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L258" t="s">
         <v>34</v>
@@ -17122,7 +17122,7 @@
         <v>34</v>
       </c>
       <c r="E260" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="F260" t="s">
         <v>242</v>
@@ -17178,7 +17178,7 @@
         <v>34</v>
       </c>
       <c r="E261" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="F261" t="s">
         <v>242</v>
@@ -17234,7 +17234,7 @@
         <v>34</v>
       </c>
       <c r="E262" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="F262" t="s">
         <v>242</v>
@@ -17264,7 +17264,7 @@
         <v>47</v>
       </c>
       <c r="O262" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="P262" t="s">
         <v>557</v>
@@ -17346,7 +17346,7 @@
         <v>34</v>
       </c>
       <c r="E264" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F264" t="s">
         <v>242</v>
@@ -17376,7 +17376,7 @@
         <v>47</v>
       </c>
       <c r="O264" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="P264" t="s">
         <v>496</v>
@@ -17570,7 +17570,7 @@
         <v>34</v>
       </c>
       <c r="E268" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="F268" t="s">
         <v>242</v>
@@ -17600,7 +17600,7 @@
         <v>47</v>
       </c>
       <c r="O268" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="P268" t="s">
         <v>561</v>
@@ -17626,7 +17626,7 @@
         <v>34</v>
       </c>
       <c r="E269" t="s">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="F269" t="s">
         <v>242</v>
@@ -17682,7 +17682,7 @@
         <v>34</v>
       </c>
       <c r="E270" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="F270" t="s">
         <v>242</v>
@@ -17738,7 +17738,7 @@
         <v>34</v>
       </c>
       <c r="E271" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F271" t="s">
         <v>242</v>
@@ -17768,7 +17768,7 @@
         <v>47</v>
       </c>
       <c r="O271" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P271" t="s">
         <v>564</v>
@@ -17794,7 +17794,7 @@
         <v>34</v>
       </c>
       <c r="E272" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="F272" t="s">
         <v>242</v>
@@ -17850,7 +17850,7 @@
         <v>34</v>
       </c>
       <c r="E273" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="F273" t="s">
         <v>242</v>
@@ -17906,7 +17906,7 @@
         <v>34</v>
       </c>
       <c r="E274" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="F274" t="s">
         <v>212</v>
@@ -17962,7 +17962,7 @@
         <v>33</v>
       </c>
       <c r="E275" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="F275" t="s">
         <v>242</v>
@@ -18018,7 +18018,7 @@
         <v>34</v>
       </c>
       <c r="E276" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="F276" t="s">
         <v>242</v>
@@ -18048,7 +18048,7 @@
         <v>47</v>
       </c>
       <c r="O276" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="P276" t="s">
         <v>502</v>
@@ -18074,7 +18074,7 @@
         <v>34</v>
       </c>
       <c r="E277" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="F277" t="s">
         <v>242</v>
@@ -18186,7 +18186,7 @@
         <v>34</v>
       </c>
       <c r="E279" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="F279" t="s">
         <v>242</v>
@@ -18216,7 +18216,7 @@
         <v>47</v>
       </c>
       <c r="O279" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="P279" t="s">
         <v>575</v>
@@ -18298,7 +18298,7 @@
         <v>34</v>
       </c>
       <c r="E281" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F281" t="s">
         <v>242</v>
@@ -18328,7 +18328,7 @@
         <v>47</v>
       </c>
       <c r="O281" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P281" t="s">
         <v>576</v>
@@ -18354,7 +18354,7 @@
         <v>34</v>
       </c>
       <c r="E282" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="F282" t="s">
         <v>242</v>
@@ -18410,7 +18410,7 @@
         <v>34</v>
       </c>
       <c r="E283" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="F283" t="s">
         <v>242</v>
@@ -18466,7 +18466,7 @@
         <v>34</v>
       </c>
       <c r="E284" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F284" t="s">
         <v>242</v>
@@ -18484,7 +18484,7 @@
         <v>189</v>
       </c>
       <c r="K284" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L284" t="s">
         <v>34</v>
@@ -19082,7 +19082,7 @@
         <v>33</v>
       </c>
       <c r="E295" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="F295" t="s">
         <v>583</v>
@@ -19138,7 +19138,7 @@
         <v>34</v>
       </c>
       <c r="E296" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="F296" t="s">
         <v>583</v>
@@ -19250,7 +19250,7 @@
         <v>34</v>
       </c>
       <c r="E298" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F298" t="s">
         <v>583</v>
@@ -19306,7 +19306,7 @@
         <v>34</v>
       </c>
       <c r="E299" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="F299" t="s">
         <v>583</v>
@@ -19321,10 +19321,10 @@
         <v>599</v>
       </c>
       <c r="J299" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="K299" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="L299" t="s">
         <v>34</v>
@@ -19362,7 +19362,7 @@
         <v>34</v>
       </c>
       <c r="E300" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="F300" t="s">
         <v>583</v>
@@ -19418,7 +19418,7 @@
         <v>34</v>
       </c>
       <c r="E301" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="F301" t="s">
         <v>583</v>
@@ -19474,7 +19474,7 @@
         <v>34</v>
       </c>
       <c r="E302" t="s">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="F302" t="s">
         <v>583</v>
@@ -19530,7 +19530,7 @@
         <v>34</v>
       </c>
       <c r="E303" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="F303" t="s">
         <v>583</v>
@@ -19866,7 +19866,7 @@
         <v>34</v>
       </c>
       <c r="E309" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="F309" t="s">
         <v>212</v>
@@ -19878,7 +19878,7 @@
         <v>608</v>
       </c>
       <c r="I309" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="J309" t="s">
         <v>70</v>
@@ -19899,7 +19899,7 @@
         <v>120</v>
       </c>
       <c r="P309" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="Q309" t="s">
         <v>47</v>
@@ -20034,7 +20034,7 @@
         <v>34</v>
       </c>
       <c r="E312" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="F312" t="s">
         <v>212</v>
@@ -20046,7 +20046,7 @@
         <v>616</v>
       </c>
       <c r="I312" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="J312" t="s">
         <v>58</v>
@@ -20064,10 +20064,10 @@
         <v>47</v>
       </c>
       <c r="O312" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="P312" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="Q312" t="s">
         <v>47</v>
@@ -20090,7 +20090,7 @@
         <v>34</v>
       </c>
       <c r="E313" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="F313" t="s">
         <v>212</v>
@@ -20120,7 +20120,7 @@
         <v>47</v>
       </c>
       <c r="O313" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="P313" t="s">
         <v>620</v>
@@ -20202,7 +20202,7 @@
         <v>34</v>
       </c>
       <c r="E315" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="F315" t="s">
         <v>242</v>
@@ -20258,7 +20258,7 @@
         <v>34</v>
       </c>
       <c r="E316" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F316" t="s">
         <v>212</v>
@@ -20273,10 +20273,10 @@
         <v>628</v>
       </c>
       <c r="J316" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="K316" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L316" t="s">
         <v>34</v>
@@ -20538,7 +20538,7 @@
         <v>33</v>
       </c>
       <c r="E321" t="s">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="F321" t="s">
         <v>212</v>
@@ -20948,7 +20948,7 @@
         <v>654</v>
       </c>
       <c r="K328" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L328" t="s">
         <v>34</v>
@@ -21016,7 +21016,7 @@
         <v>47</v>
       </c>
       <c r="O329" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P329" t="s">
         <v>657</v>
@@ -21296,7 +21296,7 @@
         <v>47</v>
       </c>
       <c r="O334" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="P334" t="s">
         <v>664</v>
@@ -21464,7 +21464,7 @@
         <v>47</v>
       </c>
       <c r="O337" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="P337" t="s">
         <v>668</v>
@@ -21564,7 +21564,7 @@
         <v>627</v>
       </c>
       <c r="K339" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L339" t="s">
         <v>34</v>
@@ -21800,7 +21800,7 @@
         <v>47</v>
       </c>
       <c r="O343" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="P343" t="s">
         <v>679</v>
@@ -22162,7 +22162,7 @@
         <v>33</v>
       </c>
       <c r="E350" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="F350" t="s">
         <v>40</v>
@@ -22218,7 +22218,7 @@
         <v>34</v>
       </c>
       <c r="E351" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F351" t="s">
         <v>40</v>
@@ -22233,10 +22233,10 @@
         <v>693</v>
       </c>
       <c r="J351" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="K351" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L351" t="s">
         <v>34</v>
@@ -22274,7 +22274,7 @@
         <v>34</v>
       </c>
       <c r="E352" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="F352" t="s">
         <v>40</v>
@@ -22386,7 +22386,7 @@
         <v>34</v>
       </c>
       <c r="E354" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F354" t="s">
         <v>694</v>
@@ -22498,7 +22498,7 @@
         <v>34</v>
       </c>
       <c r="E356" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="F356" t="s">
         <v>694</v>
@@ -22554,7 +22554,7 @@
         <v>34</v>
       </c>
       <c r="E357" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="F357" t="s">
         <v>40</v>
@@ -22584,7 +22584,7 @@
         <v>47</v>
       </c>
       <c r="O357" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="P357" t="s">
         <v>693</v>
@@ -22610,7 +22610,7 @@
         <v>34</v>
       </c>
       <c r="E358" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="F358" t="s">
         <v>40</v>
@@ -22640,7 +22640,7 @@
         <v>47</v>
       </c>
       <c r="O358" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="P358" t="s">
         <v>693</v>
@@ -22666,7 +22666,7 @@
         <v>34</v>
       </c>
       <c r="E359" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="F359" t="s">
         <v>40</v>
@@ -22834,7 +22834,7 @@
         <v>34</v>
       </c>
       <c r="E362" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="F362" t="s">
         <v>694</v>
@@ -22849,10 +22849,10 @@
         <v>693</v>
       </c>
       <c r="J362" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="K362" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="L362" t="s">
         <v>34</v>
@@ -22890,7 +22890,7 @@
         <v>34</v>
       </c>
       <c r="E363" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="F363" t="s">
         <v>40</v>
@@ -22946,7 +22946,7 @@
         <v>34</v>
       </c>
       <c r="E364" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F364" t="s">
         <v>212</v>
@@ -22976,7 +22976,7 @@
         <v>47</v>
       </c>
       <c r="O364" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P364" t="s">
         <v>692</v>
@@ -23002,7 +23002,7 @@
         <v>34</v>
       </c>
       <c r="E365" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="F365" t="s">
         <v>40</v>
@@ -23114,7 +23114,7 @@
         <v>34</v>
       </c>
       <c r="E367" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="F367" t="s">
         <v>40</v>
@@ -23200,7 +23200,7 @@
         <v>47</v>
       </c>
       <c r="O368" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P368" t="s">
         <v>692</v>
@@ -23226,7 +23226,7 @@
         <v>34</v>
       </c>
       <c r="E369" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="F369" t="s">
         <v>40</v>
@@ -23338,7 +23338,7 @@
         <v>34</v>
       </c>
       <c r="E371" t="s">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="F371" t="s">
         <v>40</v>
@@ -23394,7 +23394,7 @@
         <v>34</v>
       </c>
       <c r="E372" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="F372" t="s">
         <v>694</v>
@@ -25764,7 +25764,7 @@
         <v>195</v>
       </c>
       <c r="K414" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="L414" t="s">
         <v>34</v>
@@ -26828,7 +26828,7 @@
         <v>133</v>
       </c>
       <c r="K433" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="L433" t="s">
         <v>879</v>
@@ -28210,7 +28210,7 @@
         <v>33</v>
       </c>
       <c r="E458" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="F458" t="s">
         <v>242</v>
@@ -28266,7 +28266,7 @@
         <v>34</v>
       </c>
       <c r="E459" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="F459" t="s">
         <v>242</v>
@@ -28378,7 +28378,7 @@
         <v>34</v>
       </c>
       <c r="E461" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F461" t="s">
         <v>242</v>
@@ -28408,7 +28408,7 @@
         <v>47</v>
       </c>
       <c r="O461" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="P461" t="s">
         <v>957</v>
@@ -28434,7 +28434,7 @@
         <v>34</v>
       </c>
       <c r="E462" t="s">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="F462" t="s">
         <v>242</v>
@@ -28546,7 +28546,7 @@
         <v>34</v>
       </c>
       <c r="E464" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="F464" t="s">
         <v>242</v>
@@ -28576,7 +28576,7 @@
         <v>47</v>
       </c>
       <c r="O464" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="P464" t="s">
         <v>960</v>
@@ -28658,7 +28658,7 @@
         <v>34</v>
       </c>
       <c r="E466" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="F466" t="s">
         <v>242</v>
@@ -28688,7 +28688,7 @@
         <v>47</v>
       </c>
       <c r="O466" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="P466" t="s">
         <v>962</v>
@@ -28714,7 +28714,7 @@
         <v>34</v>
       </c>
       <c r="E467" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="F467" t="s">
         <v>242</v>
@@ -28770,7 +28770,7 @@
         <v>34</v>
       </c>
       <c r="E468" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F468" t="s">
         <v>242</v>
@@ -28800,7 +28800,7 @@
         <v>47</v>
       </c>
       <c r="O468" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="P468" t="s">
         <v>964</v>
@@ -28882,7 +28882,7 @@
         <v>34</v>
       </c>
       <c r="E470" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="F470" t="s">
         <v>242</v>
@@ -28938,7 +28938,7 @@
         <v>34</v>
       </c>
       <c r="E471" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="F471" t="s">
         <v>242</v>
@@ -28953,7 +28953,7 @@
         <v>967</v>
       </c>
       <c r="J471" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="K471" t="s">
         <v>70</v>
@@ -28968,7 +28968,7 @@
         <v>47</v>
       </c>
       <c r="O471" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="P471" t="s">
         <v>967</v>
@@ -28994,7 +28994,7 @@
         <v>34</v>
       </c>
       <c r="E472" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="F472" t="s">
         <v>242</v>
@@ -29050,7 +29050,7 @@
         <v>34</v>
       </c>
       <c r="E473" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="F473" t="s">
         <v>242</v>
@@ -29106,7 +29106,7 @@
         <v>34</v>
       </c>
       <c r="E474" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="F474" t="s">
         <v>242</v>
@@ -29162,7 +29162,7 @@
         <v>34</v>
       </c>
       <c r="E475" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F475" t="s">
         <v>242</v>
@@ -29177,10 +29177,10 @@
         <v>970</v>
       </c>
       <c r="J475" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="K475" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L475" t="s">
         <v>952</v>
@@ -29218,7 +29218,7 @@
         <v>34</v>
       </c>
       <c r="E476" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="F476" t="s">
         <v>242</v>

</xml_diff>

<commit_message>
dados: 2026-10-13 08:22 (132 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/dre/DRE_01_2026.xlsx
+++ b/xlsx/dre/DRE_01_2026.xlsx
@@ -435,13 +435,28 @@
     <t>R$  23.750,23</t>
   </si>
   <si>
+    <t>54401FIN/1</t>
+  </si>
+  <si>
+    <t>R$  24.250,23</t>
+  </si>
+  <si>
+    <t>16/01/26</t>
+  </si>
+  <si>
     <t>51101FIN/1</t>
   </si>
   <si>
     <t>R$  7.032,00</t>
   </si>
   <si>
-    <t>16/01/26</t>
+    <t>52801FIN/1</t>
+  </si>
+  <si>
+    <t>Roberta Santos de Andrade</t>
+  </si>
+  <si>
+    <t>R$  5.145,00</t>
   </si>
   <si>
     <t>55301FIN/1</t>
@@ -459,21 +474,6 @@
     <t>17/01/26</t>
   </si>
   <si>
-    <t>54401FIN/1</t>
-  </si>
-  <si>
-    <t>R$  24.250,23</t>
-  </si>
-  <si>
-    <t>52801FIN/1</t>
-  </si>
-  <si>
-    <t>Roberta Santos de Andrade</t>
-  </si>
-  <si>
-    <t>R$  5.145,00</t>
-  </si>
-  <si>
     <t>56101/0</t>
   </si>
   <si>
@@ -483,6 +483,15 @@
     <t>56101TadeuTM</t>
   </si>
   <si>
+    <t>53901FIN/1</t>
+  </si>
+  <si>
+    <t>Angelo José Valcácio Filho</t>
+  </si>
+  <si>
+    <t>R$  3.578,79</t>
+  </si>
+  <si>
     <t>53501FIN/1</t>
   </si>
   <si>
@@ -507,15 +516,6 @@
     <t>R$  24.395,47</t>
   </si>
   <si>
-    <t>53901FIN/1</t>
-  </si>
-  <si>
-    <t>Angelo José Valcácio Filho</t>
-  </si>
-  <si>
-    <t>R$  3.578,79</t>
-  </si>
-  <si>
     <t>58201FIN/1</t>
   </si>
   <si>
@@ -756,6 +756,30 @@
     <t>R$  21.103,49</t>
   </si>
   <si>
+    <t>56501/1</t>
+  </si>
+  <si>
+    <t>R$  45,51</t>
+  </si>
+  <si>
+    <t>58901/1</t>
+  </si>
+  <si>
+    <t>R$  3.866,37</t>
+  </si>
+  <si>
+    <t>55301/1</t>
+  </si>
+  <si>
+    <t>R$  6.919,66</t>
+  </si>
+  <si>
+    <t>51101/1</t>
+  </si>
+  <si>
+    <t>R$  6.708,24</t>
+  </si>
+  <si>
     <t>52201/1</t>
   </si>
   <si>
@@ -771,6 +795,18 @@
     <t>53201AnastaciaCTC</t>
   </si>
   <si>
+    <t>53901/1</t>
+  </si>
+  <si>
+    <t>R$  1.158,57</t>
+  </si>
+  <si>
+    <t>55401/1</t>
+  </si>
+  <si>
+    <t>R$  8.963,06</t>
+  </si>
+  <si>
     <t>58101/1</t>
   </si>
   <si>
@@ -795,42 +831,6 @@
     <t>R$  7.979,45</t>
   </si>
   <si>
-    <t>56501/1</t>
-  </si>
-  <si>
-    <t>R$  45,51</t>
-  </si>
-  <si>
-    <t>58901/1</t>
-  </si>
-  <si>
-    <t>R$  3.866,37</t>
-  </si>
-  <si>
-    <t>55301/1</t>
-  </si>
-  <si>
-    <t>R$  6.919,66</t>
-  </si>
-  <si>
-    <t>51101/1</t>
-  </si>
-  <si>
-    <t>R$  6.708,24</t>
-  </si>
-  <si>
-    <t>53901/1</t>
-  </si>
-  <si>
-    <t>R$  1.158,57</t>
-  </si>
-  <si>
-    <t>55401/1</t>
-  </si>
-  <si>
-    <t>R$  8.963,06</t>
-  </si>
-  <si>
     <t>54401/1</t>
   </si>
   <si>
@@ -840,13 +840,7 @@
     <t>GIR</t>
   </si>
   <si>
-    <t>53501/1</t>
-  </si>
-  <si>
-    <t>R$  1.332,44</t>
-  </si>
-  <si>
-    <t>53501CassioMMP</t>
+    <t>R$  206,07</t>
   </si>
   <si>
     <t>57201/1</t>
@@ -859,6 +853,18 @@
   </si>
   <si>
     <t>57201MarinaA</t>
+  </si>
+  <si>
+    <t>56801/1</t>
+  </si>
+  <si>
+    <t>R$  16.857,19</t>
+  </si>
+  <si>
+    <t>GiR</t>
+  </si>
+  <si>
+    <t>56801ArytanaDAST</t>
   </si>
   <si>
     <t>58201/2</t>
@@ -880,19 +886,16 @@
 </t>
   </si>
   <si>
-    <t>R$  206,07</t>
-  </si>
-  <si>
-    <t>56801/1</t>
-  </si>
-  <si>
-    <t>R$  16.857,19</t>
-  </si>
-  <si>
-    <t>GiR</t>
-  </si>
-  <si>
-    <t>56801ArytanaDAST</t>
+    <t>53501CassioMMP</t>
+  </si>
+  <si>
+    <t>53501/1</t>
+  </si>
+  <si>
+    <t>R$  1.332,44</t>
+  </si>
+  <si>
+    <t>R$  585,09</t>
   </si>
   <si>
     <t>51101/2</t>
@@ -907,9 +910,6 @@
     <t>R$  460,43</t>
   </si>
   <si>
-    <t>R$  585,09</t>
-  </si>
-  <si>
     <t>R$  4.159,95</t>
   </si>
   <si>
@@ -925,19 +925,19 @@
     <t>R$  66,29</t>
   </si>
   <si>
+    <t>R$  1.530,51</t>
+  </si>
+  <si>
+    <t>56801/0</t>
+  </si>
+  <si>
+    <t>R$  2.085,67</t>
+  </si>
+  <si>
+    <t>01/07/26</t>
+  </si>
+  <si>
     <t>R$  1.856,90</t>
-  </si>
-  <si>
-    <t>R$  1.530,51</t>
-  </si>
-  <si>
-    <t>56801/0</t>
-  </si>
-  <si>
-    <t>R$  2.085,67</t>
-  </si>
-  <si>
-    <t>01/07/26</t>
   </si>
   <si>
     <t>4.02.01.01.03 (-) Compra de mercadorias da marca - sobras</t>
@@ -5091,7 +5091,7 @@
         <v>41</v>
       </c>
       <c r="H45" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="I45" t="s">
         <v>141</v>
@@ -5100,7 +5100,7 @@
         <v>142</v>
       </c>
       <c r="K45" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L45" t="s">
         <v>84</v>
@@ -5147,16 +5147,16 @@
         <v>41</v>
       </c>
       <c r="H46" t="s">
+        <v>110</v>
+      </c>
+      <c r="I46" t="s">
         <v>144</v>
       </c>
-      <c r="I46" t="s">
-        <v>145</v>
-      </c>
       <c r="J46" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="K46" t="s">
-        <v>147</v>
+        <v>111</v>
       </c>
       <c r="L46" t="s">
         <v>84</v>
@@ -5194,7 +5194,7 @@
         <v>34</v>
       </c>
       <c r="E47" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="F47" t="s">
         <v>80</v>
@@ -5203,16 +5203,16 @@
         <v>41</v>
       </c>
       <c r="H47" t="s">
-        <v>117</v>
+        <v>146</v>
       </c>
       <c r="I47" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J47" t="s">
-        <v>142</v>
+        <v>89</v>
       </c>
       <c r="K47" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="L47" t="s">
         <v>84</v>
@@ -5250,7 +5250,7 @@
         <v>34</v>
       </c>
       <c r="E48" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F48" t="s">
         <v>80</v>
@@ -5259,16 +5259,16 @@
         <v>41</v>
       </c>
       <c r="H48" t="s">
+        <v>149</v>
+      </c>
+      <c r="I48" t="s">
+        <v>150</v>
+      </c>
+      <c r="J48" t="s">
         <v>151</v>
       </c>
-      <c r="I48" t="s">
+      <c r="K48" t="s">
         <v>152</v>
-      </c>
-      <c r="J48" t="s">
-        <v>89</v>
-      </c>
-      <c r="K48" t="s">
-        <v>133</v>
       </c>
       <c r="L48" t="s">
         <v>84</v>
@@ -5377,7 +5377,7 @@
         <v>158</v>
       </c>
       <c r="J50" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="K50" t="s">
         <v>111</v>
@@ -5421,25 +5421,25 @@
         <v>159</v>
       </c>
       <c r="F51" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G51" t="s">
         <v>41</v>
       </c>
       <c r="H51" t="s">
-        <v>86</v>
+        <v>160</v>
       </c>
       <c r="I51" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J51" t="s">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="K51" t="s">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="L51" t="s">
-        <v>34</v>
+        <v>84</v>
       </c>
       <c r="M51" t="s">
         <v>77</v>
@@ -5448,13 +5448,13 @@
         <v>47</v>
       </c>
       <c r="O51" t="s">
-        <v>161</v>
+        <v>34</v>
       </c>
       <c r="P51" t="s">
-        <v>160</v>
+        <v>34</v>
       </c>
       <c r="Q51" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R51" t="s">
         <v>34</v>
@@ -5477,25 +5477,25 @@
         <v>162</v>
       </c>
       <c r="F52" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="G52" t="s">
         <v>41</v>
       </c>
       <c r="H52" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="I52" t="s">
         <v>163</v>
       </c>
       <c r="J52" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="K52" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="L52" t="s">
-        <v>84</v>
+        <v>34</v>
       </c>
       <c r="M52" t="s">
         <v>77</v>
@@ -5504,13 +5504,13 @@
         <v>47</v>
       </c>
       <c r="O52" t="s">
-        <v>34</v>
+        <v>164</v>
       </c>
       <c r="P52" t="s">
-        <v>34</v>
+        <v>163</v>
       </c>
       <c r="Q52" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R52" t="s">
         <v>34</v>
@@ -5530,7 +5530,7 @@
         <v>34</v>
       </c>
       <c r="E53" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F53" t="s">
         <v>80</v>
@@ -5539,16 +5539,16 @@
         <v>41</v>
       </c>
       <c r="H53" t="s">
-        <v>165</v>
+        <v>95</v>
       </c>
       <c r="I53" t="s">
         <v>166</v>
       </c>
       <c r="J53" t="s">
-        <v>128</v>
+        <v>107</v>
       </c>
       <c r="K53" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="L53" t="s">
         <v>84</v>
@@ -6945,10 +6945,10 @@
         <v>248</v>
       </c>
       <c r="J78" t="s">
-        <v>97</v>
+        <v>124</v>
       </c>
       <c r="K78" t="s">
-        <v>97</v>
+        <v>124</v>
       </c>
       <c r="L78" t="s">
         <v>34</v>
@@ -6960,13 +6960,13 @@
         <v>47</v>
       </c>
       <c r="O78" t="s">
-        <v>98</v>
+        <v>34</v>
       </c>
       <c r="P78" t="s">
-        <v>248</v>
+        <v>34</v>
       </c>
       <c r="Q78" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R78" t="s">
         <v>34</v>
@@ -7001,10 +7001,10 @@
         <v>250</v>
       </c>
       <c r="J79" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="K79" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="L79" t="s">
         <v>34</v>
@@ -7016,13 +7016,13 @@
         <v>47</v>
       </c>
       <c r="O79" t="s">
-        <v>251</v>
+        <v>34</v>
       </c>
       <c r="P79" t="s">
-        <v>250</v>
+        <v>34</v>
       </c>
       <c r="Q79" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R79" t="s">
         <v>34</v>
@@ -7042,7 +7042,7 @@
         <v>34</v>
       </c>
       <c r="E80" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F80" t="s">
         <v>242</v>
@@ -7054,13 +7054,13 @@
         <v>243</v>
       </c>
       <c r="I80" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="J80" t="s">
-        <v>89</v>
+        <v>152</v>
       </c>
       <c r="K80" t="s">
-        <v>89</v>
+        <v>152</v>
       </c>
       <c r="L80" t="s">
         <v>34</v>
@@ -7098,7 +7098,7 @@
         <v>34</v>
       </c>
       <c r="E81" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F81" t="s">
         <v>242</v>
@@ -7110,13 +7110,13 @@
         <v>243</v>
       </c>
       <c r="I81" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="J81" t="s">
-        <v>70</v>
+        <v>111</v>
       </c>
       <c r="K81" t="s">
-        <v>70</v>
+        <v>111</v>
       </c>
       <c r="L81" t="s">
         <v>34</v>
@@ -7128,13 +7128,13 @@
         <v>47</v>
       </c>
       <c r="O81" t="s">
-        <v>34</v>
+        <v>112</v>
       </c>
       <c r="P81" t="s">
-        <v>34</v>
+        <v>254</v>
       </c>
       <c r="Q81" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R81" t="s">
         <v>34</v>
@@ -7154,7 +7154,7 @@
         <v>34</v>
       </c>
       <c r="E82" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F82" t="s">
         <v>242</v>
@@ -7166,13 +7166,13 @@
         <v>243</v>
       </c>
       <c r="I82" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J82" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="K82" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="L82" t="s">
         <v>34</v>
@@ -7184,13 +7184,13 @@
         <v>47</v>
       </c>
       <c r="O82" t="s">
-        <v>34</v>
+        <v>98</v>
       </c>
       <c r="P82" t="s">
-        <v>34</v>
+        <v>256</v>
       </c>
       <c r="Q82" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R82" t="s">
         <v>34</v>
@@ -7210,7 +7210,7 @@
         <v>34</v>
       </c>
       <c r="E83" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F83" t="s">
         <v>242</v>
@@ -7222,13 +7222,13 @@
         <v>243</v>
       </c>
       <c r="I83" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="J83" t="s">
-        <v>134</v>
+        <v>58</v>
       </c>
       <c r="K83" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="L83" t="s">
         <v>34</v>
@@ -7240,10 +7240,10 @@
         <v>47</v>
       </c>
       <c r="O83" t="s">
-        <v>155</v>
+        <v>259</v>
       </c>
       <c r="P83" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="Q83" t="s">
         <v>47</v>
@@ -7281,10 +7281,10 @@
         <v>261</v>
       </c>
       <c r="J84" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="K84" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="L84" t="s">
         <v>34</v>
@@ -7337,10 +7337,10 @@
         <v>263</v>
       </c>
       <c r="J85" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="K85" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="L85" t="s">
         <v>34</v>
@@ -7393,10 +7393,10 @@
         <v>265</v>
       </c>
       <c r="J86" t="s">
-        <v>147</v>
+        <v>89</v>
       </c>
       <c r="K86" t="s">
-        <v>147</v>
+        <v>89</v>
       </c>
       <c r="L86" t="s">
         <v>34</v>
@@ -7449,10 +7449,10 @@
         <v>267</v>
       </c>
       <c r="J87" t="s">
-        <v>111</v>
+        <v>70</v>
       </c>
       <c r="K87" t="s">
-        <v>111</v>
+        <v>70</v>
       </c>
       <c r="L87" t="s">
         <v>34</v>
@@ -7464,13 +7464,13 @@
         <v>47</v>
       </c>
       <c r="O87" t="s">
-        <v>112</v>
+        <v>34</v>
       </c>
       <c r="P87" t="s">
-        <v>267</v>
+        <v>34</v>
       </c>
       <c r="Q87" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R87" t="s">
         <v>34</v>
@@ -7505,10 +7505,10 @@
         <v>269</v>
       </c>
       <c r="J88" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="K88" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="L88" t="s">
         <v>34</v>
@@ -7561,10 +7561,10 @@
         <v>271</v>
       </c>
       <c r="J89" t="s">
-        <v>89</v>
+        <v>134</v>
       </c>
       <c r="K89" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="L89" t="s">
         <v>34</v>
@@ -7576,13 +7576,13 @@
         <v>47</v>
       </c>
       <c r="O89" t="s">
-        <v>34</v>
+        <v>155</v>
       </c>
       <c r="P89" t="s">
-        <v>34</v>
+        <v>271</v>
       </c>
       <c r="Q89" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R89" t="s">
         <v>34</v>
@@ -7658,7 +7658,7 @@
         <v>34</v>
       </c>
       <c r="E91" t="s">
-        <v>275</v>
+        <v>255</v>
       </c>
       <c r="F91" t="s">
         <v>212</v>
@@ -7670,13 +7670,13 @@
         <v>243</v>
       </c>
       <c r="I91" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J91" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="K91" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="L91" t="s">
         <v>34</v>
@@ -7688,10 +7688,10 @@
         <v>47</v>
       </c>
       <c r="O91" t="s">
-        <v>277</v>
+        <v>98</v>
       </c>
       <c r="P91" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="Q91" t="s">
         <v>47</v>
@@ -7714,7 +7714,7 @@
         <v>34</v>
       </c>
       <c r="E92" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="F92" t="s">
         <v>212</v>
@@ -7726,13 +7726,13 @@
         <v>243</v>
       </c>
       <c r="I92" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="J92" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="K92" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="L92" t="s">
         <v>34</v>
@@ -7744,10 +7744,10 @@
         <v>47</v>
       </c>
       <c r="O92" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="P92" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="Q92" t="s">
         <v>47</v>
@@ -7770,7 +7770,7 @@
         <v>34</v>
       </c>
       <c r="E93" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="F93" t="s">
         <v>212</v>
@@ -7782,16 +7782,16 @@
         <v>243</v>
       </c>
       <c r="I93" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J93" t="s">
-        <v>133</v>
+        <v>83</v>
       </c>
       <c r="K93" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="L93" t="s">
-        <v>34</v>
+        <v>282</v>
       </c>
       <c r="M93" t="s">
         <v>236</v>
@@ -7800,10 +7800,10 @@
         <v>47</v>
       </c>
       <c r="O93" t="s">
-        <v>214</v>
+        <v>283</v>
       </c>
       <c r="P93" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="Q93" t="s">
         <v>47</v>
@@ -7835,19 +7835,19 @@
         <v>41</v>
       </c>
       <c r="H94" t="s">
+        <v>243</v>
+      </c>
+      <c r="I94" t="s">
         <v>285</v>
       </c>
-      <c r="I94" t="s">
-        <v>286</v>
-      </c>
       <c r="J94" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="K94" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="L94" t="s">
-        <v>287</v>
+        <v>34</v>
       </c>
       <c r="M94" t="s">
         <v>236</v>
@@ -7856,10 +7856,10 @@
         <v>47</v>
       </c>
       <c r="O94" t="s">
-        <v>277</v>
+        <v>214</v>
       </c>
       <c r="P94" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="Q94" t="s">
         <v>47</v>
@@ -7882,7 +7882,7 @@
         <v>34</v>
       </c>
       <c r="E95" t="s">
-        <v>247</v>
+        <v>286</v>
       </c>
       <c r="F95" t="s">
         <v>212</v>
@@ -7891,19 +7891,19 @@
         <v>41</v>
       </c>
       <c r="H95" t="s">
-        <v>243</v>
+        <v>287</v>
       </c>
       <c r="I95" t="s">
         <v>288</v>
       </c>
       <c r="J95" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="K95" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="L95" t="s">
-        <v>34</v>
+        <v>289</v>
       </c>
       <c r="M95" t="s">
         <v>236</v>
@@ -7912,7 +7912,7 @@
         <v>47</v>
       </c>
       <c r="O95" t="s">
-        <v>98</v>
+        <v>290</v>
       </c>
       <c r="P95" t="s">
         <v>288</v>
@@ -7938,7 +7938,7 @@
         <v>34</v>
       </c>
       <c r="E96" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F96" t="s">
         <v>212</v>
@@ -7950,16 +7950,16 @@
         <v>243</v>
       </c>
       <c r="I96" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="J96" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="K96" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L96" t="s">
-        <v>291</v>
+        <v>34</v>
       </c>
       <c r="M96" t="s">
         <v>236</v>
@@ -7968,10 +7968,10 @@
         <v>47</v>
       </c>
       <c r="O96" t="s">
+        <v>290</v>
+      </c>
+      <c r="P96" t="s">
         <v>292</v>
-      </c>
-      <c r="P96" t="s">
-        <v>290</v>
       </c>
       <c r="Q96" t="s">
         <v>47</v>
@@ -7994,7 +7994,7 @@
         <v>34</v>
       </c>
       <c r="E97" t="s">
-        <v>293</v>
+        <v>241</v>
       </c>
       <c r="F97" t="s">
         <v>212</v>
@@ -8006,13 +8006,13 @@
         <v>243</v>
       </c>
       <c r="I97" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J97" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="K97" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="L97" t="s">
         <v>34</v>
@@ -8024,10 +8024,10 @@
         <v>47</v>
       </c>
       <c r="O97" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="P97" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="Q97" t="s">
         <v>47</v>
@@ -8050,7 +8050,7 @@
         <v>34</v>
       </c>
       <c r="E98" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F98" t="s">
         <v>212</v>
@@ -8062,13 +8062,13 @@
         <v>243</v>
       </c>
       <c r="I98" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J98" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="K98" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L98" t="s">
         <v>34</v>
@@ -8080,10 +8080,10 @@
         <v>47</v>
       </c>
       <c r="O98" t="s">
-        <v>292</v>
+        <v>112</v>
       </c>
       <c r="P98" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="Q98" t="s">
         <v>47</v>
@@ -8106,7 +8106,7 @@
         <v>34</v>
       </c>
       <c r="E99" t="s">
-        <v>241</v>
+        <v>296</v>
       </c>
       <c r="F99" t="s">
         <v>212</v>
@@ -8121,10 +8121,10 @@
         <v>297</v>
       </c>
       <c r="J99" t="s">
-        <v>128</v>
+        <v>83</v>
       </c>
       <c r="K99" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="L99" t="s">
         <v>34</v>
@@ -8136,7 +8136,7 @@
         <v>47</v>
       </c>
       <c r="O99" t="s">
-        <v>103</v>
+        <v>283</v>
       </c>
       <c r="P99" t="s">
         <v>297</v>
@@ -8162,7 +8162,7 @@
         <v>34</v>
       </c>
       <c r="E100" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="F100" t="s">
         <v>212</v>
@@ -8171,7 +8171,7 @@
         <v>41</v>
       </c>
       <c r="H100" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="I100" t="s">
         <v>298</v>
@@ -8192,7 +8192,7 @@
         <v>47</v>
       </c>
       <c r="O100" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P100" t="s">
         <v>298</v>
@@ -8248,7 +8248,7 @@
         <v>47</v>
       </c>
       <c r="O101" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P101" t="s">
         <v>300</v>
@@ -8330,7 +8330,7 @@
         <v>34</v>
       </c>
       <c r="E103" t="s">
-        <v>245</v>
+        <v>109</v>
       </c>
       <c r="F103" t="s">
         <v>212</v>
@@ -8339,7 +8339,7 @@
         <v>41</v>
       </c>
       <c r="H103" t="s">
-        <v>243</v>
+        <v>287</v>
       </c>
       <c r="I103" t="s">
         <v>303</v>
@@ -8348,7 +8348,7 @@
         <v>70</v>
       </c>
       <c r="K103" t="s">
-        <v>70</v>
+        <v>111</v>
       </c>
       <c r="L103" t="s">
         <v>34</v>
@@ -8360,7 +8360,7 @@
         <v>47</v>
       </c>
       <c r="O103" t="s">
-        <v>173</v>
+        <v>112</v>
       </c>
       <c r="P103" t="s">
         <v>303</v>
@@ -8386,7 +8386,7 @@
         <v>34</v>
       </c>
       <c r="E104" t="s">
-        <v>109</v>
+        <v>304</v>
       </c>
       <c r="F104" t="s">
         <v>212</v>
@@ -8395,16 +8395,16 @@
         <v>41</v>
       </c>
       <c r="H104" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="I104" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="J104" t="s">
-        <v>70</v>
+        <v>306</v>
       </c>
       <c r="K104" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L104" t="s">
         <v>34</v>
@@ -8416,10 +8416,10 @@
         <v>47</v>
       </c>
       <c r="O104" t="s">
-        <v>112</v>
+        <v>283</v>
       </c>
       <c r="P104" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="Q104" t="s">
         <v>47</v>
@@ -8442,7 +8442,7 @@
         <v>34</v>
       </c>
       <c r="E105" t="s">
-        <v>305</v>
+        <v>245</v>
       </c>
       <c r="F105" t="s">
         <v>212</v>
@@ -8451,16 +8451,16 @@
         <v>41</v>
       </c>
       <c r="H105" t="s">
-        <v>285</v>
+        <v>243</v>
       </c>
       <c r="I105" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J105" t="s">
-        <v>307</v>
+        <v>70</v>
       </c>
       <c r="K105" t="s">
-        <v>119</v>
+        <v>70</v>
       </c>
       <c r="L105" t="s">
         <v>34</v>
@@ -8472,10 +8472,10 @@
         <v>47</v>
       </c>
       <c r="O105" t="s">
-        <v>292</v>
+        <v>173</v>
       </c>
       <c r="P105" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Q105" t="s">
         <v>47</v>
@@ -10096,7 +10096,7 @@
         <v>47</v>
       </c>
       <c r="O134" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="P134" t="s">
         <v>385</v>
@@ -10137,10 +10137,10 @@
         <v>387</v>
       </c>
       <c r="J135" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="K135" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="L135" t="s">
         <v>361</v>
@@ -10152,7 +10152,7 @@
         <v>47</v>
       </c>
       <c r="O135" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="P135" t="s">
         <v>387</v>
@@ -10178,7 +10178,7 @@
         <v>34</v>
       </c>
       <c r="E136" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="F136" t="s">
         <v>242</v>
@@ -10208,7 +10208,7 @@
         <v>47</v>
       </c>
       <c r="O136" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="P136" t="s">
         <v>385</v>
@@ -10305,10 +10305,10 @@
         <v>390</v>
       </c>
       <c r="J138" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="K138" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="L138" t="s">
         <v>361</v>
@@ -10320,7 +10320,7 @@
         <v>47</v>
       </c>
       <c r="O138" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="P138" t="s">
         <v>390</v>
@@ -10417,10 +10417,10 @@
         <v>394</v>
       </c>
       <c r="J140" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="K140" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L140" t="s">
         <v>361</v>
@@ -10529,10 +10529,10 @@
         <v>399</v>
       </c>
       <c r="J142" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="K142" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L142" t="s">
         <v>361</v>
@@ -10600,7 +10600,7 @@
         <v>47</v>
       </c>
       <c r="O143" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P143" t="s">
         <v>401</v>
@@ -10656,7 +10656,7 @@
         <v>47</v>
       </c>
       <c r="O144" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P144" t="s">
         <v>403</v>
@@ -10824,7 +10824,7 @@
         <v>47</v>
       </c>
       <c r="O147" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P147" t="s">
         <v>408</v>
@@ -10962,7 +10962,7 @@
         <v>34</v>
       </c>
       <c r="E150" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F150" t="s">
         <v>242</v>
@@ -11074,7 +11074,7 @@
         <v>34</v>
       </c>
       <c r="E152" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F152" t="s">
         <v>242</v>
@@ -11104,7 +11104,7 @@
         <v>47</v>
       </c>
       <c r="O152" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P152" t="s">
         <v>415</v>
@@ -11130,7 +11130,7 @@
         <v>34</v>
       </c>
       <c r="E153" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="F153" t="s">
         <v>242</v>
@@ -11858,7 +11858,7 @@
         <v>34</v>
       </c>
       <c r="E166" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F166" t="s">
         <v>212</v>
@@ -11888,7 +11888,7 @@
         <v>47</v>
       </c>
       <c r="O166" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P166" t="s">
         <v>443</v>
@@ -11932,7 +11932,7 @@
         <v>442</v>
       </c>
       <c r="K167" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L167" t="s">
         <v>34</v>
@@ -12041,10 +12041,10 @@
         <v>450</v>
       </c>
       <c r="J169" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="K169" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L169" t="s">
         <v>34</v>
@@ -12138,7 +12138,7 @@
         <v>34</v>
       </c>
       <c r="E171" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F171" t="s">
         <v>212</v>
@@ -12168,7 +12168,7 @@
         <v>47</v>
       </c>
       <c r="O171" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P171" t="s">
         <v>453</v>
@@ -12209,10 +12209,10 @@
         <v>454</v>
       </c>
       <c r="J172" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="K172" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L172" t="s">
         <v>34</v>
@@ -12380,7 +12380,7 @@
         <v>442</v>
       </c>
       <c r="K175" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L175" t="s">
         <v>34</v>
@@ -12616,7 +12616,7 @@
         <v>47</v>
       </c>
       <c r="O179" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P179" t="s">
         <v>464</v>
@@ -12840,7 +12840,7 @@
         <v>47</v>
       </c>
       <c r="O183" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P183" t="s">
         <v>470</v>
@@ -13426,7 +13426,7 @@
         <v>33</v>
       </c>
       <c r="E194" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="F194" t="s">
         <v>242</v>
@@ -13538,7 +13538,7 @@
         <v>34</v>
       </c>
       <c r="E196" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="F196" t="s">
         <v>242</v>
@@ -13650,7 +13650,7 @@
         <v>34</v>
       </c>
       <c r="E198" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="F198" t="s">
         <v>242</v>
@@ -13706,7 +13706,7 @@
         <v>34</v>
       </c>
       <c r="E199" t="s">
-        <v>266</v>
+        <v>253</v>
       </c>
       <c r="F199" t="s">
         <v>242</v>
@@ -13818,7 +13818,7 @@
         <v>34</v>
       </c>
       <c r="E201" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="F201" t="s">
         <v>242</v>
@@ -13874,7 +13874,7 @@
         <v>34</v>
       </c>
       <c r="E202" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="F202" t="s">
         <v>242</v>
@@ -13904,7 +13904,7 @@
         <v>47</v>
       </c>
       <c r="O202" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="P202" t="s">
         <v>496</v>
@@ -13930,7 +13930,7 @@
         <v>34</v>
       </c>
       <c r="E203" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="F203" t="s">
         <v>242</v>
@@ -13986,7 +13986,7 @@
         <v>34</v>
       </c>
       <c r="E204" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
       <c r="F204" t="s">
         <v>242</v>
@@ -14004,7 +14004,7 @@
         <v>189</v>
       </c>
       <c r="K204" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L204" t="s">
         <v>34</v>
@@ -14042,7 +14042,7 @@
         <v>34</v>
       </c>
       <c r="E205" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="F205" t="s">
         <v>242</v>
@@ -14098,7 +14098,7 @@
         <v>34</v>
       </c>
       <c r="E206" t="s">
-        <v>275</v>
+        <v>291</v>
       </c>
       <c r="F206" t="s">
         <v>242</v>
@@ -14128,7 +14128,7 @@
         <v>47</v>
       </c>
       <c r="O206" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="P206" t="s">
         <v>502</v>
@@ -14154,7 +14154,7 @@
         <v>34</v>
       </c>
       <c r="E207" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="F207" t="s">
         <v>242</v>
@@ -14184,7 +14184,7 @@
         <v>47</v>
       </c>
       <c r="O207" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P207" t="s">
         <v>503</v>
@@ -14210,7 +14210,7 @@
         <v>34</v>
       </c>
       <c r="E208" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="F208" t="s">
         <v>242</v>
@@ -14378,7 +14378,7 @@
         <v>34</v>
       </c>
       <c r="E211" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="F211" t="s">
         <v>242</v>
@@ -14408,7 +14408,7 @@
         <v>47</v>
       </c>
       <c r="O211" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P211" t="s">
         <v>509</v>
@@ -14490,7 +14490,7 @@
         <v>33</v>
       </c>
       <c r="E213" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="F213" t="s">
         <v>242</v>
@@ -14658,7 +14658,7 @@
         <v>34</v>
       </c>
       <c r="E216" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="F216" t="s">
         <v>242</v>
@@ -14688,7 +14688,7 @@
         <v>47</v>
       </c>
       <c r="O216" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="P216" t="s">
         <v>518</v>
@@ -14714,7 +14714,7 @@
         <v>34</v>
       </c>
       <c r="E217" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="F217" t="s">
         <v>242</v>
@@ -14770,7 +14770,7 @@
         <v>34</v>
       </c>
       <c r="E218" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="F218" t="s">
         <v>242</v>
@@ -14800,7 +14800,7 @@
         <v>47</v>
       </c>
       <c r="O218" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P218" t="s">
         <v>520</v>
@@ -14826,7 +14826,7 @@
         <v>34</v>
       </c>
       <c r="E219" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="F219" t="s">
         <v>242</v>
@@ -14856,7 +14856,7 @@
         <v>47</v>
       </c>
       <c r="O219" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="P219" t="s">
         <v>522</v>
@@ -14882,7 +14882,7 @@
         <v>34</v>
       </c>
       <c r="E220" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="F220" t="s">
         <v>242</v>
@@ -14912,7 +14912,7 @@
         <v>47</v>
       </c>
       <c r="O220" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="P220" t="s">
         <v>525</v>
@@ -14938,7 +14938,7 @@
         <v>34</v>
       </c>
       <c r="E221" t="s">
-        <v>275</v>
+        <v>291</v>
       </c>
       <c r="F221" t="s">
         <v>242</v>
@@ -14968,7 +14968,7 @@
         <v>47</v>
       </c>
       <c r="O221" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="P221" t="s">
         <v>527</v>
@@ -14994,7 +14994,7 @@
         <v>34</v>
       </c>
       <c r="E222" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="F222" t="s">
         <v>242</v>
@@ -15050,7 +15050,7 @@
         <v>34</v>
       </c>
       <c r="E223" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="F223" t="s">
         <v>242</v>
@@ -15080,7 +15080,7 @@
         <v>47</v>
       </c>
       <c r="O223" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P223" t="s">
         <v>529</v>
@@ -15106,7 +15106,7 @@
         <v>34</v>
       </c>
       <c r="E224" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="F224" t="s">
         <v>242</v>
@@ -15274,7 +15274,7 @@
         <v>34</v>
       </c>
       <c r="E227" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="F227" t="s">
         <v>242</v>
@@ -15304,7 +15304,7 @@
         <v>47</v>
       </c>
       <c r="O227" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P227" t="s">
         <v>533</v>
@@ -15386,7 +15386,7 @@
         <v>34</v>
       </c>
       <c r="E229" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="F229" t="s">
         <v>242</v>
@@ -15498,7 +15498,7 @@
         <v>34</v>
       </c>
       <c r="E231" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="F231" t="s">
         <v>242</v>
@@ -15554,7 +15554,7 @@
         <v>34</v>
       </c>
       <c r="E232" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="F232" t="s">
         <v>242</v>
@@ -15610,7 +15610,7 @@
         <v>34</v>
       </c>
       <c r="E233" t="s">
-        <v>266</v>
+        <v>253</v>
       </c>
       <c r="F233" t="s">
         <v>242</v>
@@ -15666,7 +15666,7 @@
         <v>34</v>
       </c>
       <c r="E234" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
       <c r="F234" t="s">
         <v>242</v>
@@ -15684,7 +15684,7 @@
         <v>189</v>
       </c>
       <c r="K234" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L234" t="s">
         <v>34</v>
@@ -15778,7 +15778,7 @@
         <v>34</v>
       </c>
       <c r="E236" t="s">
-        <v>266</v>
+        <v>253</v>
       </c>
       <c r="F236" t="s">
         <v>242</v>
@@ -15946,7 +15946,7 @@
         <v>34</v>
       </c>
       <c r="E239" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
       <c r="F239" t="s">
         <v>242</v>
@@ -15964,7 +15964,7 @@
         <v>341</v>
       </c>
       <c r="K239" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L239" t="s">
         <v>34</v>
@@ -16058,7 +16058,7 @@
         <v>34</v>
       </c>
       <c r="E241" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="F241" t="s">
         <v>242</v>
@@ -16114,7 +16114,7 @@
         <v>34</v>
       </c>
       <c r="E242" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="F242" t="s">
         <v>242</v>
@@ -16144,7 +16144,7 @@
         <v>47</v>
       </c>
       <c r="O242" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P242" t="s">
         <v>549</v>
@@ -16170,7 +16170,7 @@
         <v>34</v>
       </c>
       <c r="E243" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="F243" t="s">
         <v>242</v>
@@ -16200,7 +16200,7 @@
         <v>47</v>
       </c>
       <c r="O243" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="P243" t="s">
         <v>550</v>
@@ -16226,7 +16226,7 @@
         <v>34</v>
       </c>
       <c r="E244" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="F244" t="s">
         <v>242</v>
@@ -16282,7 +16282,7 @@
         <v>34</v>
       </c>
       <c r="E245" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="F245" t="s">
         <v>242</v>
@@ -16338,7 +16338,7 @@
         <v>34</v>
       </c>
       <c r="E246" t="s">
-        <v>275</v>
+        <v>291</v>
       </c>
       <c r="F246" t="s">
         <v>242</v>
@@ -16368,7 +16368,7 @@
         <v>47</v>
       </c>
       <c r="O246" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="P246" t="s">
         <v>553</v>
@@ -16394,7 +16394,7 @@
         <v>34</v>
       </c>
       <c r="E247" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="F247" t="s">
         <v>242</v>
@@ -16450,7 +16450,7 @@
         <v>34</v>
       </c>
       <c r="E248" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="F248" t="s">
         <v>242</v>
@@ -16480,7 +16480,7 @@
         <v>47</v>
       </c>
       <c r="O248" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P248" t="s">
         <v>509</v>
@@ -16506,7 +16506,7 @@
         <v>34</v>
       </c>
       <c r="E249" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="F249" t="s">
         <v>242</v>
@@ -16562,7 +16562,7 @@
         <v>34</v>
       </c>
       <c r="E250" t="s">
-        <v>260</v>
+        <v>247</v>
       </c>
       <c r="F250" t="s">
         <v>242</v>
@@ -16618,7 +16618,7 @@
         <v>34</v>
       </c>
       <c r="E251" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="F251" t="s">
         <v>242</v>
@@ -16674,7 +16674,7 @@
         <v>34</v>
       </c>
       <c r="E252" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="F252" t="s">
         <v>242</v>
@@ -16704,7 +16704,7 @@
         <v>47</v>
       </c>
       <c r="O252" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P252" t="s">
         <v>503</v>
@@ -16730,7 +16730,7 @@
         <v>34</v>
       </c>
       <c r="E253" t="s">
-        <v>275</v>
+        <v>291</v>
       </c>
       <c r="F253" t="s">
         <v>242</v>
@@ -16760,7 +16760,7 @@
         <v>47</v>
       </c>
       <c r="O253" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="P253" t="s">
         <v>502</v>
@@ -16786,7 +16786,7 @@
         <v>34</v>
       </c>
       <c r="E254" t="s">
-        <v>266</v>
+        <v>253</v>
       </c>
       <c r="F254" t="s">
         <v>242</v>
@@ -16842,7 +16842,7 @@
         <v>34</v>
       </c>
       <c r="E255" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="F255" t="s">
         <v>242</v>
@@ -16898,7 +16898,7 @@
         <v>34</v>
       </c>
       <c r="E256" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="F256" t="s">
         <v>242</v>
@@ -17010,7 +17010,7 @@
         <v>34</v>
       </c>
       <c r="E258" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
       <c r="F258" t="s">
         <v>242</v>
@@ -17028,7 +17028,7 @@
         <v>189</v>
       </c>
       <c r="K258" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L258" t="s">
         <v>34</v>
@@ -17122,7 +17122,7 @@
         <v>34</v>
       </c>
       <c r="E260" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="F260" t="s">
         <v>242</v>
@@ -17234,7 +17234,7 @@
         <v>34</v>
       </c>
       <c r="E262" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="F262" t="s">
         <v>242</v>
@@ -17264,7 +17264,7 @@
         <v>47</v>
       </c>
       <c r="O262" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="P262" t="s">
         <v>557</v>
@@ -17290,7 +17290,7 @@
         <v>34</v>
       </c>
       <c r="E263" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="F263" t="s">
         <v>242</v>
@@ -17346,7 +17346,7 @@
         <v>34</v>
       </c>
       <c r="E264" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="F264" t="s">
         <v>242</v>
@@ -17376,7 +17376,7 @@
         <v>47</v>
       </c>
       <c r="O264" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="P264" t="s">
         <v>496</v>
@@ -17514,7 +17514,7 @@
         <v>34</v>
       </c>
       <c r="E267" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="F267" t="s">
         <v>242</v>
@@ -17570,7 +17570,7 @@
         <v>34</v>
       </c>
       <c r="E268" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="F268" t="s">
         <v>242</v>
@@ -17600,7 +17600,7 @@
         <v>47</v>
       </c>
       <c r="O268" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="P268" t="s">
         <v>561</v>
@@ -17626,7 +17626,7 @@
         <v>34</v>
       </c>
       <c r="E269" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="F269" t="s">
         <v>242</v>
@@ -17682,7 +17682,7 @@
         <v>34</v>
       </c>
       <c r="E270" t="s">
-        <v>260</v>
+        <v>247</v>
       </c>
       <c r="F270" t="s">
         <v>242</v>
@@ -17738,7 +17738,7 @@
         <v>34</v>
       </c>
       <c r="E271" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="F271" t="s">
         <v>242</v>
@@ -17768,7 +17768,7 @@
         <v>47</v>
       </c>
       <c r="O271" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P271" t="s">
         <v>564</v>
@@ -17794,7 +17794,7 @@
         <v>34</v>
       </c>
       <c r="E272" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="F272" t="s">
         <v>242</v>
@@ -17850,7 +17850,7 @@
         <v>34</v>
       </c>
       <c r="E273" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="F273" t="s">
         <v>242</v>
@@ -17906,7 +17906,7 @@
         <v>34</v>
       </c>
       <c r="E274" t="s">
-        <v>260</v>
+        <v>247</v>
       </c>
       <c r="F274" t="s">
         <v>212</v>
@@ -17962,7 +17962,7 @@
         <v>33</v>
       </c>
       <c r="E275" t="s">
-        <v>266</v>
+        <v>253</v>
       </c>
       <c r="F275" t="s">
         <v>242</v>
@@ -18018,7 +18018,7 @@
         <v>34</v>
       </c>
       <c r="E276" t="s">
-        <v>275</v>
+        <v>291</v>
       </c>
       <c r="F276" t="s">
         <v>242</v>
@@ -18048,7 +18048,7 @@
         <v>47</v>
       </c>
       <c r="O276" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="P276" t="s">
         <v>502</v>
@@ -18186,7 +18186,7 @@
         <v>34</v>
       </c>
       <c r="E279" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="F279" t="s">
         <v>242</v>
@@ -18216,7 +18216,7 @@
         <v>47</v>
       </c>
       <c r="O279" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P279" t="s">
         <v>575</v>
@@ -18298,7 +18298,7 @@
         <v>34</v>
       </c>
       <c r="E281" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="F281" t="s">
         <v>242</v>
@@ -18328,7 +18328,7 @@
         <v>47</v>
       </c>
       <c r="O281" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P281" t="s">
         <v>576</v>
@@ -18354,7 +18354,7 @@
         <v>34</v>
       </c>
       <c r="E282" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="F282" t="s">
         <v>242</v>
@@ -18466,7 +18466,7 @@
         <v>34</v>
       </c>
       <c r="E284" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
       <c r="F284" t="s">
         <v>242</v>
@@ -18484,7 +18484,7 @@
         <v>189</v>
       </c>
       <c r="K284" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L284" t="s">
         <v>34</v>
@@ -19082,7 +19082,7 @@
         <v>33</v>
       </c>
       <c r="E295" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="F295" t="s">
         <v>583</v>
@@ -19138,7 +19138,7 @@
         <v>34</v>
       </c>
       <c r="E296" t="s">
-        <v>266</v>
+        <v>253</v>
       </c>
       <c r="F296" t="s">
         <v>583</v>
@@ -19250,7 +19250,7 @@
         <v>34</v>
       </c>
       <c r="E298" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="F298" t="s">
         <v>583</v>
@@ -19306,7 +19306,7 @@
         <v>34</v>
       </c>
       <c r="E299" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="F299" t="s">
         <v>583</v>
@@ -19321,10 +19321,10 @@
         <v>599</v>
       </c>
       <c r="J299" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="K299" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="L299" t="s">
         <v>34</v>
@@ -19362,7 +19362,7 @@
         <v>34</v>
       </c>
       <c r="E300" t="s">
-        <v>260</v>
+        <v>247</v>
       </c>
       <c r="F300" t="s">
         <v>583</v>
@@ -19418,7 +19418,7 @@
         <v>34</v>
       </c>
       <c r="E301" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="F301" t="s">
         <v>583</v>
@@ -19474,7 +19474,7 @@
         <v>34</v>
       </c>
       <c r="E302" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="F302" t="s">
         <v>583</v>
@@ -19530,7 +19530,7 @@
         <v>34</v>
       </c>
       <c r="E303" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="F303" t="s">
         <v>583</v>
@@ -19878,7 +19878,7 @@
         <v>608</v>
       </c>
       <c r="I309" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="J309" t="s">
         <v>70</v>
@@ -19899,7 +19899,7 @@
         <v>120</v>
       </c>
       <c r="P309" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="Q309" t="s">
         <v>47</v>
@@ -19978,7 +19978,7 @@
         <v>34</v>
       </c>
       <c r="E311" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="F311" t="s">
         <v>583</v>
@@ -20034,7 +20034,7 @@
         <v>34</v>
       </c>
       <c r="E312" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="F312" t="s">
         <v>212</v>
@@ -20046,7 +20046,7 @@
         <v>616</v>
       </c>
       <c r="I312" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="J312" t="s">
         <v>58</v>
@@ -20064,10 +20064,10 @@
         <v>47</v>
       </c>
       <c r="O312" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P312" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="Q312" t="s">
         <v>47</v>
@@ -20090,7 +20090,7 @@
         <v>34</v>
       </c>
       <c r="E313" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="F313" t="s">
         <v>212</v>
@@ -20120,7 +20120,7 @@
         <v>47</v>
       </c>
       <c r="O313" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P313" t="s">
         <v>620</v>
@@ -20202,7 +20202,7 @@
         <v>34</v>
       </c>
       <c r="E315" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="F315" t="s">
         <v>242</v>
@@ -20258,7 +20258,7 @@
         <v>34</v>
       </c>
       <c r="E316" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
       <c r="F316" t="s">
         <v>212</v>
@@ -20273,10 +20273,10 @@
         <v>628</v>
       </c>
       <c r="J316" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="K316" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L316" t="s">
         <v>34</v>
@@ -20538,7 +20538,7 @@
         <v>33</v>
       </c>
       <c r="E321" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="F321" t="s">
         <v>212</v>
@@ -20948,7 +20948,7 @@
         <v>654</v>
       </c>
       <c r="K328" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L328" t="s">
         <v>34</v>
@@ -20986,7 +20986,7 @@
         <v>34</v>
       </c>
       <c r="E329" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F329" t="s">
         <v>212</v>
@@ -21016,7 +21016,7 @@
         <v>47</v>
       </c>
       <c r="O329" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P329" t="s">
         <v>657</v>
@@ -21296,7 +21296,7 @@
         <v>47</v>
       </c>
       <c r="O334" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P334" t="s">
         <v>664</v>
@@ -21464,7 +21464,7 @@
         <v>47</v>
       </c>
       <c r="O337" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P337" t="s">
         <v>668</v>
@@ -21564,7 +21564,7 @@
         <v>627</v>
       </c>
       <c r="K339" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L339" t="s">
         <v>34</v>
@@ -21800,7 +21800,7 @@
         <v>47</v>
       </c>
       <c r="O343" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="P343" t="s">
         <v>679</v>
@@ -22162,7 +22162,7 @@
         <v>33</v>
       </c>
       <c r="E350" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="F350" t="s">
         <v>40</v>
@@ -22218,7 +22218,7 @@
         <v>34</v>
       </c>
       <c r="E351" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
       <c r="F351" t="s">
         <v>40</v>
@@ -22233,10 +22233,10 @@
         <v>693</v>
       </c>
       <c r="J351" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="K351" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L351" t="s">
         <v>34</v>
@@ -22274,7 +22274,7 @@
         <v>34</v>
       </c>
       <c r="E352" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="F352" t="s">
         <v>40</v>
@@ -22386,7 +22386,7 @@
         <v>34</v>
       </c>
       <c r="E354" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="F354" t="s">
         <v>694</v>
@@ -22498,7 +22498,7 @@
         <v>34</v>
       </c>
       <c r="E356" t="s">
-        <v>260</v>
+        <v>247</v>
       </c>
       <c r="F356" t="s">
         <v>694</v>
@@ -22554,7 +22554,7 @@
         <v>34</v>
       </c>
       <c r="E357" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="F357" t="s">
         <v>40</v>
@@ -22584,7 +22584,7 @@
         <v>47</v>
       </c>
       <c r="O357" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P357" t="s">
         <v>693</v>
@@ -22610,7 +22610,7 @@
         <v>34</v>
       </c>
       <c r="E358" t="s">
-        <v>275</v>
+        <v>291</v>
       </c>
       <c r="F358" t="s">
         <v>40</v>
@@ -22640,7 +22640,7 @@
         <v>47</v>
       </c>
       <c r="O358" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="P358" t="s">
         <v>693</v>
@@ -22666,7 +22666,7 @@
         <v>34</v>
       </c>
       <c r="E359" t="s">
-        <v>266</v>
+        <v>253</v>
       </c>
       <c r="F359" t="s">
         <v>40</v>
@@ -22722,7 +22722,7 @@
         <v>34</v>
       </c>
       <c r="E360" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="F360" t="s">
         <v>694</v>
@@ -22834,7 +22834,7 @@
         <v>34</v>
       </c>
       <c r="E362" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="F362" t="s">
         <v>694</v>
@@ -22849,10 +22849,10 @@
         <v>693</v>
       </c>
       <c r="J362" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="K362" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="L362" t="s">
         <v>34</v>
@@ -22890,7 +22890,7 @@
         <v>34</v>
       </c>
       <c r="E363" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="F363" t="s">
         <v>40</v>
@@ -22946,7 +22946,7 @@
         <v>34</v>
       </c>
       <c r="E364" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="F364" t="s">
         <v>212</v>
@@ -22976,7 +22976,7 @@
         <v>47</v>
       </c>
       <c r="O364" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P364" t="s">
         <v>692</v>
@@ -23114,7 +23114,7 @@
         <v>34</v>
       </c>
       <c r="E367" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="F367" t="s">
         <v>40</v>
@@ -23170,7 +23170,7 @@
         <v>34</v>
       </c>
       <c r="E368" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F368" t="s">
         <v>212</v>
@@ -23200,7 +23200,7 @@
         <v>47</v>
       </c>
       <c r="O368" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P368" t="s">
         <v>692</v>
@@ -23338,7 +23338,7 @@
         <v>34</v>
       </c>
       <c r="E371" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="F371" t="s">
         <v>40</v>
@@ -23394,7 +23394,7 @@
         <v>34</v>
       </c>
       <c r="E372" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="F372" t="s">
         <v>694</v>
@@ -25764,7 +25764,7 @@
         <v>195</v>
       </c>
       <c r="K414" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="L414" t="s">
         <v>34</v>
@@ -26828,7 +26828,7 @@
         <v>133</v>
       </c>
       <c r="K433" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="L433" t="s">
         <v>879</v>
@@ -28210,7 +28210,7 @@
         <v>33</v>
       </c>
       <c r="E458" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="F458" t="s">
         <v>242</v>
@@ -28266,7 +28266,7 @@
         <v>34</v>
       </c>
       <c r="E459" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="F459" t="s">
         <v>242</v>
@@ -28378,7 +28378,7 @@
         <v>34</v>
       </c>
       <c r="E461" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="F461" t="s">
         <v>242</v>
@@ -28408,7 +28408,7 @@
         <v>47</v>
       </c>
       <c r="O461" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="P461" t="s">
         <v>957</v>
@@ -28434,7 +28434,7 @@
         <v>34</v>
       </c>
       <c r="E462" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="F462" t="s">
         <v>242</v>
@@ -28546,7 +28546,7 @@
         <v>34</v>
       </c>
       <c r="E464" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="F464" t="s">
         <v>242</v>
@@ -28576,7 +28576,7 @@
         <v>47</v>
       </c>
       <c r="O464" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P464" t="s">
         <v>960</v>
@@ -28658,7 +28658,7 @@
         <v>34</v>
       </c>
       <c r="E466" t="s">
-        <v>275</v>
+        <v>291</v>
       </c>
       <c r="F466" t="s">
         <v>242</v>
@@ -28688,7 +28688,7 @@
         <v>47</v>
       </c>
       <c r="O466" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="P466" t="s">
         <v>962</v>
@@ -28714,7 +28714,7 @@
         <v>34</v>
       </c>
       <c r="E467" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="F467" t="s">
         <v>242</v>
@@ -28770,7 +28770,7 @@
         <v>34</v>
       </c>
       <c r="E468" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="F468" t="s">
         <v>242</v>
@@ -28800,7 +28800,7 @@
         <v>47</v>
       </c>
       <c r="O468" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="P468" t="s">
         <v>964</v>
@@ -28826,7 +28826,7 @@
         <v>34</v>
       </c>
       <c r="E469" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="F469" t="s">
         <v>242</v>
@@ -28882,7 +28882,7 @@
         <v>34</v>
       </c>
       <c r="E470" t="s">
-        <v>266</v>
+        <v>253</v>
       </c>
       <c r="F470" t="s">
         <v>242</v>
@@ -28938,7 +28938,7 @@
         <v>34</v>
       </c>
       <c r="E471" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="F471" t="s">
         <v>242</v>
@@ -28953,7 +28953,7 @@
         <v>967</v>
       </c>
       <c r="J471" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="K471" t="s">
         <v>70</v>
@@ -28968,7 +28968,7 @@
         <v>47</v>
       </c>
       <c r="O471" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="P471" t="s">
         <v>967</v>
@@ -29050,7 +29050,7 @@
         <v>34</v>
       </c>
       <c r="E473" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="F473" t="s">
         <v>242</v>
@@ -29162,7 +29162,7 @@
         <v>34</v>
       </c>
       <c r="E475" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
       <c r="F475" t="s">
         <v>242</v>
@@ -29177,10 +29177,10 @@
         <v>970</v>
       </c>
       <c r="J475" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="K475" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="L475" t="s">
         <v>952</v>
@@ -29218,7 +29218,7 @@
         <v>34</v>
       </c>
       <c r="E476" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="F476" t="s">
         <v>242</v>

</xml_diff>

<commit_message>
dados: 2026-10-15 08:20 (132 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/dre/DRE_01_2026.xlsx
+++ b/xlsx/dre/DRE_01_2026.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9904" uniqueCount="1083">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9904" uniqueCount="1084">
   <si>
     <t>Movimentações Financeiras</t>
   </si>
@@ -2273,6 +2273,9 @@
   </si>
   <si>
     <t>Rubens - Pagamento 2026</t>
+  </si>
+  <si>
+    <t>CARINA PEREIRA</t>
   </si>
   <si>
     <t>R$  2.090,00</t>
@@ -24414,10 +24417,10 @@
         <v>41</v>
       </c>
       <c r="H390" t="s">
-        <v>524</v>
+        <v>750</v>
       </c>
       <c r="I390" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="J390" t="s">
         <v>97</v>
@@ -24426,7 +24429,7 @@
         <v>45</v>
       </c>
       <c r="L390" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="M390" t="s">
         <v>744</v>
@@ -24438,7 +24441,7 @@
         <v>48</v>
       </c>
       <c r="P390" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="Q390" t="s">
         <v>47</v>
@@ -24470,10 +24473,10 @@
         <v>41</v>
       </c>
       <c r="H391" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="I391" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="J391" t="s">
         <v>97</v>
@@ -24482,7 +24485,7 @@
         <v>45</v>
       </c>
       <c r="L391" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="M391" t="s">
         <v>744</v>
@@ -24494,7 +24497,7 @@
         <v>48</v>
       </c>
       <c r="P391" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="Q391" t="s">
         <v>47</v>
@@ -24529,7 +24532,7 @@
         <v>513</v>
       </c>
       <c r="I392" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="J392" t="s">
         <v>341</v>
@@ -24538,7 +24541,7 @@
         <v>45</v>
       </c>
       <c r="L392" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="M392" t="s">
         <v>744</v>
@@ -24550,7 +24553,7 @@
         <v>48</v>
       </c>
       <c r="P392" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="Q392" t="s">
         <v>47</v>
@@ -24582,10 +24585,10 @@
         <v>41</v>
       </c>
       <c r="H393" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="I393" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="J393" t="s">
         <v>97</v>
@@ -24594,7 +24597,7 @@
         <v>45</v>
       </c>
       <c r="L393" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="M393" t="s">
         <v>744</v>
@@ -24606,7 +24609,7 @@
         <v>48</v>
       </c>
       <c r="P393" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="Q393" t="s">
         <v>47</v>
@@ -24638,10 +24641,10 @@
         <v>41</v>
       </c>
       <c r="H394" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="I394" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="J394" t="s">
         <v>341</v>
@@ -24650,7 +24653,7 @@
         <v>102</v>
       </c>
       <c r="L394" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="M394" t="s">
         <v>744</v>
@@ -24662,7 +24665,7 @@
         <v>48</v>
       </c>
       <c r="P394" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="Q394" t="s">
         <v>47</v>
@@ -24694,10 +24697,10 @@
         <v>41</v>
       </c>
       <c r="H395" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="I395" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="J395" t="s">
         <v>58</v>
@@ -24706,7 +24709,7 @@
         <v>45</v>
       </c>
       <c r="L395" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="M395" t="s">
         <v>744</v>
@@ -24718,7 +24721,7 @@
         <v>48</v>
       </c>
       <c r="P395" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="Q395" t="s">
         <v>47</v>
@@ -24750,10 +24753,10 @@
         <v>41</v>
       </c>
       <c r="H396" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="I396" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="J396" t="s">
         <v>97</v>
@@ -24762,7 +24765,7 @@
         <v>45</v>
       </c>
       <c r="L396" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="M396" t="s">
         <v>744</v>
@@ -24774,7 +24777,7 @@
         <v>48</v>
       </c>
       <c r="P396" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="Q396" t="s">
         <v>47</v>
@@ -24806,10 +24809,10 @@
         <v>41</v>
       </c>
       <c r="H397" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="I397" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="J397" t="s">
         <v>97</v>
@@ -24818,7 +24821,7 @@
         <v>45</v>
       </c>
       <c r="L397" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="M397" t="s">
         <v>744</v>
@@ -24830,7 +24833,7 @@
         <v>48</v>
       </c>
       <c r="P397" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="Q397" t="s">
         <v>47</v>
@@ -24853,7 +24856,7 @@
         <v>34</v>
       </c>
       <c r="E398" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="F398" t="s">
         <v>212</v>
@@ -24897,13 +24900,13 @@
     </row>
     <row r="399">
       <c r="A399" t="s" s="1">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="B399" t="s" s="1">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="C399" t="s" s="1">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="D399" t="s" s="1">
         <v>33</v>
@@ -24953,13 +24956,13 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
+        <v>774</v>
+      </c>
+      <c r="B400" t="s">
         <v>773</v>
       </c>
-      <c r="B400" t="s">
-        <v>772</v>
-      </c>
       <c r="C400" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="D400" t="s">
         <v>33</v>
@@ -24986,10 +24989,10 @@
         <v>115</v>
       </c>
       <c r="L400" t="s">
+        <v>775</v>
+      </c>
+      <c r="M400" t="s">
         <v>774</v>
-      </c>
-      <c r="M400" t="s">
-        <v>773</v>
       </c>
       <c r="N400" t="s">
         <v>47</v>
@@ -25009,13 +25012,13 @@
     </row>
     <row r="401">
       <c r="A401" t="s" s="1">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="B401" t="s" s="1">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="C401" t="s" s="1">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="D401" t="s" s="1">
         <v>33</v>
@@ -25065,13 +25068,13 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
+        <v>778</v>
+      </c>
+      <c r="B402" t="s">
         <v>777</v>
       </c>
-      <c r="B402" t="s">
-        <v>776</v>
-      </c>
       <c r="C402" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="D402" t="s">
         <v>33</v>
@@ -25098,10 +25101,10 @@
         <v>115</v>
       </c>
       <c r="L402" t="s">
+        <v>779</v>
+      </c>
+      <c r="M402" t="s">
         <v>778</v>
-      </c>
-      <c r="M402" t="s">
-        <v>777</v>
       </c>
       <c r="N402" t="s">
         <v>47</v>
@@ -25121,13 +25124,13 @@
     </row>
     <row r="403">
       <c r="A403" t="s" s="1">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="B403" t="s" s="1">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="C403" t="s" s="1">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="D403" t="s" s="1">
         <v>33</v>
@@ -25177,13 +25180,13 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
+        <v>782</v>
+      </c>
+      <c r="B404" t="s">
         <v>781</v>
       </c>
-      <c r="B404" t="s">
-        <v>780</v>
-      </c>
       <c r="C404" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="D404" t="s">
         <v>33</v>
@@ -25198,10 +25201,10 @@
         <v>41</v>
       </c>
       <c r="H404" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="I404" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="J404" t="s">
         <v>115</v>
@@ -25210,10 +25213,10 @@
         <v>115</v>
       </c>
       <c r="L404" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="M404" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="N404" t="s">
         <v>47</v>
@@ -25222,7 +25225,7 @@
         <v>48</v>
       </c>
       <c r="P404" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="Q404" t="s">
         <v>47</v>
@@ -25233,13 +25236,13 @@
     </row>
     <row r="405">
       <c r="A405" t="s" s="1">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="B405" t="s" s="1">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="C405" t="s" s="1">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="D405" t="s" s="1">
         <v>33</v>
@@ -25289,13 +25292,13 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
+        <v>788</v>
+      </c>
+      <c r="B406" t="s">
         <v>787</v>
       </c>
-      <c r="B406" t="s">
-        <v>786</v>
-      </c>
       <c r="C406" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="D406" t="s">
         <v>33</v>
@@ -25313,7 +25316,7 @@
         <v>578</v>
       </c>
       <c r="I406" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="J406" t="s">
         <v>115</v>
@@ -25325,7 +25328,7 @@
         <v>34</v>
       </c>
       <c r="M406" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="N406" t="s">
         <v>47</v>
@@ -25345,13 +25348,13 @@
     </row>
     <row r="407">
       <c r="A407" t="s" s="1">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="B407" t="s" s="1">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="C407" t="s" s="1">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="D407" t="s" s="1">
         <v>33</v>
@@ -25401,13 +25404,13 @@
     </row>
     <row r="408">
       <c r="A408" t="s" s="1">
+        <v>792</v>
+      </c>
+      <c r="B408" t="s" s="1">
         <v>791</v>
       </c>
-      <c r="B408" t="s" s="1">
-        <v>790</v>
-      </c>
       <c r="C408" t="s" s="1">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="D408" t="s" s="1">
         <v>33</v>
@@ -25457,19 +25460,19 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="B409" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="C409" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="D409" t="s">
         <v>33</v>
       </c>
       <c r="E409" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="F409" t="s">
         <v>40</v>
@@ -25481,7 +25484,7 @@
         <v>540</v>
       </c>
       <c r="I409" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="J409" t="s">
         <v>729</v>
@@ -25490,10 +25493,10 @@
         <v>718</v>
       </c>
       <c r="L409" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="M409" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="N409" t="s">
         <v>47</v>
@@ -25502,7 +25505,7 @@
         <v>48</v>
       </c>
       <c r="P409" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="Q409" t="s">
         <v>47</v>
@@ -25513,7 +25516,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="B410" t="s">
         <v>34</v>
@@ -25525,7 +25528,7 @@
         <v>34</v>
       </c>
       <c r="E410" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="F410" t="s">
         <v>212</v>
@@ -25537,10 +25540,10 @@
         <v>485</v>
       </c>
       <c r="I410" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="J410" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="K410" t="s">
         <v>325</v>
@@ -25549,7 +25552,7 @@
         <v>34</v>
       </c>
       <c r="M410" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="N410" t="s">
         <v>47</v>
@@ -25558,7 +25561,7 @@
         <v>48</v>
       </c>
       <c r="P410" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="Q410" t="s">
         <v>47</v>
@@ -25569,13 +25572,13 @@
     </row>
     <row r="411">
       <c r="A411" t="s" s="1">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="B411" t="s" s="1">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="C411" t="s" s="1">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="D411" t="s" s="1">
         <v>33</v>
@@ -25625,13 +25628,13 @@
     </row>
     <row r="412">
       <c r="A412" t="s" s="1">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="B412" t="s" s="1">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="C412" t="s" s="1">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="D412" t="s" s="1">
         <v>33</v>
@@ -25681,19 +25684,19 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="B413" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="C413" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="D413" t="s">
         <v>33</v>
       </c>
       <c r="E413" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="F413" t="s">
         <v>212</v>
@@ -25702,10 +25705,10 @@
         <v>41</v>
       </c>
       <c r="H413" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="I413" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="J413" t="s">
         <v>730</v>
@@ -25717,7 +25720,7 @@
         <v>34</v>
       </c>
       <c r="M413" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="N413" t="s">
         <v>47</v>
@@ -25726,7 +25729,7 @@
         <v>48</v>
       </c>
       <c r="P413" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="Q413" t="s">
         <v>47</v>
@@ -25737,19 +25740,19 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="B414" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="C414" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="D414" t="s">
         <v>33</v>
       </c>
       <c r="E414" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="F414" t="s">
         <v>212</v>
@@ -25761,7 +25764,7 @@
         <v>193</v>
       </c>
       <c r="I414" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="J414" t="s">
         <v>195</v>
@@ -25773,7 +25776,7 @@
         <v>34</v>
       </c>
       <c r="M414" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="N414" t="s">
         <v>47</v>
@@ -25782,7 +25785,7 @@
         <v>48</v>
       </c>
       <c r="P414" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="Q414" t="s">
         <v>47</v>
@@ -25793,13 +25796,13 @@
     </row>
     <row r="415">
       <c r="A415" t="s" s="1">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="B415" t="s" s="1">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="C415" t="s" s="1">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="D415" t="s" s="1">
         <v>33</v>
@@ -25849,19 +25852,19 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
+        <v>815</v>
+      </c>
+      <c r="B416" t="s">
         <v>814</v>
       </c>
-      <c r="B416" t="s">
-        <v>813</v>
-      </c>
       <c r="C416" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="D416" t="s">
         <v>33</v>
       </c>
       <c r="E416" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="F416" t="s">
         <v>40</v>
@@ -25870,10 +25873,10 @@
         <v>41</v>
       </c>
       <c r="H416" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="I416" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="J416" t="s">
         <v>124</v>
@@ -25882,10 +25885,10 @@
         <v>312</v>
       </c>
       <c r="L416" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="M416" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="N416" t="s">
         <v>47</v>
@@ -25894,7 +25897,7 @@
         <v>48</v>
       </c>
       <c r="P416" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="Q416" t="s">
         <v>47</v>
@@ -25905,13 +25908,13 @@
     </row>
     <row r="417">
       <c r="A417" t="s" s="1">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="B417" t="s" s="1">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="C417" t="s" s="1">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="D417" t="s" s="1">
         <v>33</v>
@@ -25961,13 +25964,13 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
+        <v>822</v>
+      </c>
+      <c r="B418" t="s">
         <v>821</v>
       </c>
-      <c r="B418" t="s">
-        <v>820</v>
-      </c>
       <c r="C418" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="D418" t="s">
         <v>33</v>
@@ -25982,10 +25985,10 @@
         <v>41</v>
       </c>
       <c r="H418" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="I418" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="J418" t="s">
         <v>97</v>
@@ -25994,10 +25997,10 @@
         <v>45</v>
       </c>
       <c r="L418" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="M418" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="N418" t="s">
         <v>47</v>
@@ -26006,7 +26009,7 @@
         <v>48</v>
       </c>
       <c r="P418" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="Q418" t="s">
         <v>47</v>
@@ -26017,13 +26020,13 @@
     </row>
     <row r="419">
       <c r="A419" t="s" s="1">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="B419" t="s" s="1">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="C419" t="s" s="1">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="D419" t="s" s="1">
         <v>33</v>
@@ -26073,19 +26076,19 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="B420" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="C420" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="D420" t="s">
         <v>33</v>
       </c>
       <c r="E420" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="F420" t="s">
         <v>40</v>
@@ -26094,22 +26097,22 @@
         <v>41</v>
       </c>
       <c r="H420" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="I420" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="J420" t="s">
         <v>133</v>
       </c>
       <c r="K420" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="L420" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="M420" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="N420" t="s">
         <v>47</v>
@@ -26118,7 +26121,7 @@
         <v>48</v>
       </c>
       <c r="P420" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="Q420" t="s">
         <v>47</v>
@@ -26129,13 +26132,13 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="B421" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="C421" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="D421" t="s">
         <v>33</v>
@@ -26150,10 +26153,10 @@
         <v>41</v>
       </c>
       <c r="H421" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="I421" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="J421" t="s">
         <v>97</v>
@@ -26162,10 +26165,10 @@
         <v>730</v>
       </c>
       <c r="L421" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="M421" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="N421" t="s">
         <v>47</v>
@@ -26174,7 +26177,7 @@
         <v>48</v>
       </c>
       <c r="P421" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="Q421" t="s">
         <v>47</v>
@@ -26185,13 +26188,13 @@
     </row>
     <row r="422">
       <c r="A422" t="s" s="1">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="B422" t="s" s="1">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="C422" t="s" s="1">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="D422" t="s" s="1">
         <v>33</v>
@@ -26241,19 +26244,19 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
+        <v>840</v>
+      </c>
+      <c r="B423" t="s">
         <v>839</v>
       </c>
-      <c r="B423" t="s">
-        <v>838</v>
-      </c>
       <c r="C423" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="D423" t="s">
         <v>33</v>
       </c>
       <c r="E423" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="F423" t="s">
         <v>40</v>
@@ -26262,22 +26265,22 @@
         <v>41</v>
       </c>
       <c r="H423" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="I423" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="J423" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="K423" t="s">
         <v>718</v>
       </c>
       <c r="L423" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="M423" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="N423" t="s">
         <v>47</v>
@@ -26286,7 +26289,7 @@
         <v>48</v>
       </c>
       <c r="P423" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="Q423" t="s">
         <v>47</v>
@@ -26297,13 +26300,13 @@
     </row>
     <row r="424">
       <c r="A424" t="s" s="1">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="B424" t="s" s="1">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="C424" t="s" s="1">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="D424" t="s" s="1">
         <v>33</v>
@@ -26353,19 +26356,19 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
+        <v>848</v>
+      </c>
+      <c r="B425" t="s">
         <v>847</v>
       </c>
-      <c r="B425" t="s">
-        <v>846</v>
-      </c>
       <c r="C425" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="D425" t="s">
         <v>33</v>
       </c>
       <c r="E425" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="F425" t="s">
         <v>212</v>
@@ -26374,10 +26377,10 @@
         <v>41</v>
       </c>
       <c r="H425" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="I425" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="J425" t="s">
         <v>341</v>
@@ -26386,10 +26389,10 @@
         <v>128</v>
       </c>
       <c r="L425" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="M425" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="N425" t="s">
         <v>47</v>
@@ -26398,7 +26401,7 @@
         <v>48</v>
       </c>
       <c r="P425" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="Q425" t="s">
         <v>47</v>
@@ -26409,7 +26412,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="B426" t="s">
         <v>34</v>
@@ -26421,7 +26424,7 @@
         <v>34</v>
       </c>
       <c r="E426" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F426" t="s">
         <v>212</v>
@@ -26430,10 +26433,10 @@
         <v>41</v>
       </c>
       <c r="H426" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="I426" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="J426" t="s">
         <v>341</v>
@@ -26442,10 +26445,10 @@
         <v>128</v>
       </c>
       <c r="L426" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="M426" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="N426" t="s">
         <v>47</v>
@@ -26454,7 +26457,7 @@
         <v>48</v>
       </c>
       <c r="P426" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="Q426" t="s">
         <v>47</v>
@@ -26465,7 +26468,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="B427" t="s">
         <v>34</v>
@@ -26477,7 +26480,7 @@
         <v>34</v>
       </c>
       <c r="E427" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="F427" t="s">
         <v>212</v>
@@ -26486,10 +26489,10 @@
         <v>41</v>
       </c>
       <c r="H427" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="I427" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="J427" t="s">
         <v>341</v>
@@ -26501,7 +26504,7 @@
         <v>34</v>
       </c>
       <c r="M427" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="N427" t="s">
         <v>47</v>
@@ -26510,7 +26513,7 @@
         <v>48</v>
       </c>
       <c r="P427" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="Q427" t="s">
         <v>47</v>
@@ -26521,7 +26524,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="B428" t="s">
         <v>34</v>
@@ -26533,7 +26536,7 @@
         <v>34</v>
       </c>
       <c r="E428" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="F428" t="s">
         <v>212</v>
@@ -26545,7 +26548,7 @@
         <v>56</v>
       </c>
       <c r="I428" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="J428" t="s">
         <v>341</v>
@@ -26554,10 +26557,10 @@
         <v>325</v>
       </c>
       <c r="L428" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="M428" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="N428" t="s">
         <v>47</v>
@@ -26566,7 +26569,7 @@
         <v>48</v>
       </c>
       <c r="P428" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="Q428" t="s">
         <v>47</v>
@@ -26577,7 +26580,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="B429" t="s">
         <v>34</v>
@@ -26589,7 +26592,7 @@
         <v>34</v>
       </c>
       <c r="E429" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="F429" t="s">
         <v>212</v>
@@ -26598,10 +26601,10 @@
         <v>41</v>
       </c>
       <c r="H429" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="I429" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="J429" t="s">
         <v>341</v>
@@ -26610,10 +26613,10 @@
         <v>119</v>
       </c>
       <c r="L429" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="M429" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="N429" t="s">
         <v>47</v>
@@ -26622,7 +26625,7 @@
         <v>48</v>
       </c>
       <c r="P429" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="Q429" t="s">
         <v>47</v>
@@ -26633,7 +26636,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="B430" t="s">
         <v>34</v>
@@ -26645,7 +26648,7 @@
         <v>34</v>
       </c>
       <c r="E430" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="F430" t="s">
         <v>212</v>
@@ -26654,10 +26657,10 @@
         <v>41</v>
       </c>
       <c r="H430" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="I430" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="J430" t="s">
         <v>89</v>
@@ -26666,10 +26669,10 @@
         <v>89</v>
       </c>
       <c r="L430" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="M430" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="N430" t="s">
         <v>47</v>
@@ -26678,7 +26681,7 @@
         <v>48</v>
       </c>
       <c r="P430" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="Q430" t="s">
         <v>47</v>
@@ -26689,13 +26692,13 @@
     </row>
     <row r="431">
       <c r="A431" t="s" s="1">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="B431" t="s" s="1">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="C431" t="s" s="1">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="D431" t="s" s="1">
         <v>33</v>
@@ -26745,13 +26748,13 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="B432" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="C432" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="D432" t="s">
         <v>33</v>
@@ -26766,10 +26769,10 @@
         <v>41</v>
       </c>
       <c r="H432" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="I432" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="J432" t="s">
         <v>97</v>
@@ -26778,10 +26781,10 @@
         <v>45</v>
       </c>
       <c r="L432" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="M432" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="N432" t="s">
         <v>47</v>
@@ -26790,7 +26793,7 @@
         <v>48</v>
       </c>
       <c r="P432" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="Q432" t="s">
         <v>47</v>
@@ -26801,19 +26804,19 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="B433" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="C433" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="D433" t="s">
         <v>33</v>
       </c>
       <c r="E433" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="F433" t="s">
         <v>40</v>
@@ -26822,10 +26825,10 @@
         <v>41</v>
       </c>
       <c r="H433" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="I433" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="J433" t="s">
         <v>133</v>
@@ -26834,10 +26837,10 @@
         <v>151</v>
       </c>
       <c r="L433" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="M433" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="N433" t="s">
         <v>47</v>
@@ -26846,7 +26849,7 @@
         <v>48</v>
       </c>
       <c r="P433" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="Q433" t="s">
         <v>47</v>
@@ -26857,19 +26860,19 @@
     </row>
     <row r="434">
       <c r="A434" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="B434" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="C434" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="D434" t="s">
         <v>33</v>
       </c>
       <c r="E434" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="F434" t="s">
         <v>40</v>
@@ -26878,10 +26881,10 @@
         <v>41</v>
       </c>
       <c r="H434" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="I434" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="J434" t="s">
         <v>44</v>
@@ -26890,10 +26893,10 @@
         <v>45</v>
       </c>
       <c r="L434" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="M434" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="N434" t="s">
         <v>47</v>
@@ -26902,7 +26905,7 @@
         <v>48</v>
       </c>
       <c r="P434" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="Q434" t="s">
         <v>47</v>
@@ -26913,13 +26916,13 @@
     </row>
     <row r="435">
       <c r="A435" t="s" s="1">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="B435" t="s" s="1">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="C435" t="s" s="1">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="D435" t="s" s="1">
         <v>33</v>
@@ -26969,19 +26972,19 @@
     </row>
     <row r="436">
       <c r="A436" t="s">
+        <v>889</v>
+      </c>
+      <c r="B436" t="s">
         <v>888</v>
       </c>
-      <c r="B436" t="s">
-        <v>887</v>
-      </c>
       <c r="C436" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="D436" t="s">
         <v>33</v>
       </c>
       <c r="E436" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="F436" t="s">
         <v>212</v>
@@ -26990,10 +26993,10 @@
         <v>41</v>
       </c>
       <c r="H436" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="I436" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="J436" t="s">
         <v>341</v>
@@ -27005,7 +27008,7 @@
         <v>34</v>
       </c>
       <c r="M436" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="N436" t="s">
         <v>47</v>
@@ -27014,7 +27017,7 @@
         <v>48</v>
       </c>
       <c r="P436" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="Q436" t="s">
         <v>47</v>
@@ -27025,7 +27028,7 @@
     </row>
     <row r="437">
       <c r="A437" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="B437" t="s">
         <v>34</v>
@@ -27037,7 +27040,7 @@
         <v>34</v>
       </c>
       <c r="E437" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="F437" t="s">
         <v>40</v>
@@ -27046,10 +27049,10 @@
         <v>41</v>
       </c>
       <c r="H437" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="I437" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="J437" t="s">
         <v>58</v>
@@ -27058,10 +27061,10 @@
         <v>97</v>
       </c>
       <c r="L437" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="M437" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="N437" t="s">
         <v>47</v>
@@ -27070,7 +27073,7 @@
         <v>48</v>
       </c>
       <c r="P437" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="Q437" t="s">
         <v>47</v>
@@ -27081,7 +27084,7 @@
     </row>
     <row r="438">
       <c r="A438" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="B438" t="s">
         <v>34</v>
@@ -27093,7 +27096,7 @@
         <v>34</v>
       </c>
       <c r="E438" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="F438" t="s">
         <v>40</v>
@@ -27102,10 +27105,10 @@
         <v>41</v>
       </c>
       <c r="H438" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="I438" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="J438" t="s">
         <v>341</v>
@@ -27114,10 +27117,10 @@
         <v>45</v>
       </c>
       <c r="L438" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="M438" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="N438" t="s">
         <v>47</v>
@@ -27126,7 +27129,7 @@
         <v>48</v>
       </c>
       <c r="P438" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="Q438" t="s">
         <v>47</v>
@@ -27137,7 +27140,7 @@
     </row>
     <row r="439">
       <c r="A439" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="B439" t="s">
         <v>34</v>
@@ -27158,10 +27161,10 @@
         <v>41</v>
       </c>
       <c r="H439" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="I439" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="J439" t="s">
         <v>58</v>
@@ -27170,10 +27173,10 @@
         <v>97</v>
       </c>
       <c r="L439" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="M439" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="N439" t="s">
         <v>47</v>
@@ -27182,7 +27185,7 @@
         <v>48</v>
       </c>
       <c r="P439" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="Q439" t="s">
         <v>47</v>
@@ -27193,7 +27196,7 @@
     </row>
     <row r="440">
       <c r="A440" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="B440" t="s">
         <v>34</v>
@@ -27214,10 +27217,10 @@
         <v>41</v>
       </c>
       <c r="H440" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="I440" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="J440" t="s">
         <v>58</v>
@@ -27226,10 +27229,10 @@
         <v>45</v>
       </c>
       <c r="L440" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="M440" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="N440" t="s">
         <v>47</v>
@@ -27238,7 +27241,7 @@
         <v>48</v>
       </c>
       <c r="P440" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="Q440" t="s">
         <v>47</v>
@@ -27249,13 +27252,13 @@
     </row>
     <row r="441">
       <c r="A441" t="s" s="1">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="B441" t="s" s="1">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="C441" t="s" s="1">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="D441" t="s" s="1">
         <v>33</v>
@@ -27305,19 +27308,19 @@
     </row>
     <row r="442">
       <c r="A442" t="s">
+        <v>906</v>
+      </c>
+      <c r="B442" t="s">
         <v>905</v>
       </c>
-      <c r="B442" t="s">
-        <v>904</v>
-      </c>
       <c r="C442" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="D442" t="s">
         <v>33</v>
       </c>
       <c r="E442" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="F442" t="s">
         <v>212</v>
@@ -27329,7 +27332,7 @@
         <v>56</v>
       </c>
       <c r="I442" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="J442" t="s">
         <v>341</v>
@@ -27338,10 +27341,10 @@
         <v>196</v>
       </c>
       <c r="L442" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="M442" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="N442" t="s">
         <v>47</v>
@@ -27350,7 +27353,7 @@
         <v>48</v>
       </c>
       <c r="P442" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="Q442" t="s">
         <v>47</v>
@@ -27361,7 +27364,7 @@
     </row>
     <row r="443">
       <c r="A443" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="B443" t="s">
         <v>34</v>
@@ -27373,7 +27376,7 @@
         <v>34</v>
       </c>
       <c r="E443" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="F443" t="s">
         <v>212</v>
@@ -27382,10 +27385,10 @@
         <v>41</v>
       </c>
       <c r="H443" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="I443" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="J443" t="s">
         <v>58</v>
@@ -27397,7 +27400,7 @@
         <v>34</v>
       </c>
       <c r="M443" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="N443" t="s">
         <v>47</v>
@@ -27406,7 +27409,7 @@
         <v>48</v>
       </c>
       <c r="P443" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="Q443" t="s">
         <v>47</v>
@@ -27417,13 +27420,13 @@
     </row>
     <row r="444">
       <c r="A444" t="s" s="1">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="B444" t="s" s="1">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="C444" t="s" s="1">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="D444" t="s" s="1">
         <v>33</v>
@@ -27473,13 +27476,13 @@
     </row>
     <row r="445">
       <c r="A445" t="s">
+        <v>915</v>
+      </c>
+      <c r="B445" t="s">
         <v>914</v>
       </c>
-      <c r="B445" t="s">
-        <v>913</v>
-      </c>
       <c r="C445" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="D445" t="s">
         <v>33</v>
@@ -27494,10 +27497,10 @@
         <v>41</v>
       </c>
       <c r="H445" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="I445" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="J445" t="s">
         <v>97</v>
@@ -27506,10 +27509,10 @@
         <v>45</v>
       </c>
       <c r="L445" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="M445" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="N445" t="s">
         <v>47</v>
@@ -27518,7 +27521,7 @@
         <v>48</v>
       </c>
       <c r="P445" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="Q445" t="s">
         <v>47</v>
@@ -27529,13 +27532,13 @@
     </row>
     <row r="446">
       <c r="A446" t="s" s="1">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="B446" t="s" s="1">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="C446" t="s" s="1">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="D446" t="s" s="1">
         <v>33</v>
@@ -27585,13 +27588,13 @@
     </row>
     <row r="447">
       <c r="A447" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="B447" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="C447" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="D447" t="s">
         <v>33</v>
@@ -27606,10 +27609,10 @@
         <v>41</v>
       </c>
       <c r="H447" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="I447" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="J447" t="s">
         <v>115</v>
@@ -27618,10 +27621,10 @@
         <v>111</v>
       </c>
       <c r="L447" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="M447" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="N447" t="s">
         <v>47</v>
@@ -27630,7 +27633,7 @@
         <v>48</v>
       </c>
       <c r="P447" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="Q447" t="s">
         <v>47</v>
@@ -27641,19 +27644,19 @@
     </row>
     <row r="448">
       <c r="A448" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="B448" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="C448" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="D448" t="s">
         <v>33</v>
       </c>
       <c r="E448" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="F448" t="s">
         <v>40</v>
@@ -27662,10 +27665,10 @@
         <v>41</v>
       </c>
       <c r="H448" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
       <c r="I448" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="J448" t="s">
         <v>337</v>
@@ -27674,10 +27677,10 @@
         <v>205</v>
       </c>
       <c r="L448" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="M448" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="N448" t="s">
         <v>47</v>
@@ -27686,7 +27689,7 @@
         <v>48</v>
       </c>
       <c r="P448" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="Q448" t="s">
         <v>47</v>
@@ -27697,7 +27700,7 @@
     </row>
     <row r="449">
       <c r="A449" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="B449" t="s">
         <v>34</v>
@@ -27718,7 +27721,7 @@
         <v>41</v>
       </c>
       <c r="H449" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="I449" t="s">
         <v>693</v>
@@ -27730,10 +27733,10 @@
         <v>45</v>
       </c>
       <c r="L449" t="s">
-        <v>932</v>
+        <v>933</v>
       </c>
       <c r="M449" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="N449" t="s">
         <v>47</v>
@@ -27753,13 +27756,13 @@
     </row>
     <row r="450">
       <c r="A450" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="B450" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="C450" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="D450" t="s">
         <v>33</v>
@@ -27774,10 +27777,10 @@
         <v>41</v>
       </c>
       <c r="H450" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="I450" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="J450" t="s">
         <v>45</v>
@@ -27786,10 +27789,10 @@
         <v>45</v>
       </c>
       <c r="L450" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
       <c r="M450" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="N450" t="s">
         <v>47</v>
@@ -27798,7 +27801,7 @@
         <v>48</v>
       </c>
       <c r="P450" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="Q450" t="s">
         <v>47</v>
@@ -27809,13 +27812,13 @@
     </row>
     <row r="451">
       <c r="A451" t="s" s="1">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="B451" t="s" s="1">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="C451" t="s" s="1">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="D451" t="s" s="1">
         <v>33</v>
@@ -27865,13 +27868,13 @@
     </row>
     <row r="452">
       <c r="A452" t="s" s="1">
+        <v>941</v>
+      </c>
+      <c r="B452" t="s" s="1">
         <v>940</v>
       </c>
-      <c r="B452" t="s" s="1">
-        <v>939</v>
-      </c>
       <c r="C452" t="s" s="1">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="D452" t="s" s="1">
         <v>33</v>
@@ -27921,13 +27924,13 @@
     </row>
     <row r="453">
       <c r="A453" t="s" s="1">
-        <v>941</v>
+        <v>942</v>
       </c>
       <c r="B453" t="s" s="1">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="C453" t="s" s="1">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="D453" t="s" s="1">
         <v>33</v>
@@ -27977,19 +27980,19 @@
     </row>
     <row r="454">
       <c r="A454" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="B454" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="C454" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="D454" t="s">
         <v>33</v>
       </c>
       <c r="E454" t="s">
-        <v>943</v>
+        <v>944</v>
       </c>
       <c r="F454" t="s">
         <v>212</v>
@@ -27998,10 +28001,10 @@
         <v>41</v>
       </c>
       <c r="H454" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="I454" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="J454" t="s">
         <v>341</v>
@@ -28013,7 +28016,7 @@
         <v>34</v>
       </c>
       <c r="M454" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="N454" t="s">
         <v>47</v>
@@ -28022,7 +28025,7 @@
         <v>48</v>
       </c>
       <c r="P454" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="Q454" t="s">
         <v>47</v>
@@ -28033,13 +28036,13 @@
     </row>
     <row r="455">
       <c r="A455" t="s" s="1">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="B455" t="s" s="1">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="C455" t="s" s="1">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="D455" t="s" s="1">
         <v>33</v>
@@ -28089,13 +28092,13 @@
     </row>
     <row r="456">
       <c r="A456" t="s" s="1">
+        <v>949</v>
+      </c>
+      <c r="B456" t="s" s="1">
         <v>948</v>
       </c>
-      <c r="B456" t="s" s="1">
-        <v>947</v>
-      </c>
       <c r="C456" t="s" s="1">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="D456" t="s" s="1">
         <v>33</v>
@@ -28145,13 +28148,13 @@
     </row>
     <row r="457">
       <c r="A457" t="s" s="1">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="B457" t="s" s="1">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="C457" t="s" s="1">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="D457" t="s" s="1">
         <v>33</v>
@@ -28201,13 +28204,13 @@
     </row>
     <row r="458">
       <c r="A458" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B458" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="C458" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="D458" t="s">
         <v>33</v>
@@ -28222,10 +28225,10 @@
         <v>41</v>
       </c>
       <c r="H458" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I458" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="J458" t="s">
         <v>111</v>
@@ -28234,19 +28237,19 @@
         <v>111</v>
       </c>
       <c r="L458" t="s">
+        <v>954</v>
+      </c>
+      <c r="M458" t="s">
+        <v>951</v>
+      </c>
+      <c r="N458" t="s">
+        <v>47</v>
+      </c>
+      <c r="O458" t="s">
+        <v>955</v>
+      </c>
+      <c r="P458" t="s">
         <v>953</v>
-      </c>
-      <c r="M458" t="s">
-        <v>950</v>
-      </c>
-      <c r="N458" t="s">
-        <v>47</v>
-      </c>
-      <c r="O458" t="s">
-        <v>954</v>
-      </c>
-      <c r="P458" t="s">
-        <v>952</v>
       </c>
       <c r="Q458" t="s">
         <v>47</v>
@@ -28257,7 +28260,7 @@
     </row>
     <row r="459">
       <c r="A459" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B459" t="s">
         <v>34</v>
@@ -28278,10 +28281,10 @@
         <v>41</v>
       </c>
       <c r="H459" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I459" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="J459" t="s">
         <v>97</v>
@@ -28290,10 +28293,10 @@
         <v>97</v>
       </c>
       <c r="L459" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M459" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N459" t="s">
         <v>47</v>
@@ -28302,7 +28305,7 @@
         <v>98</v>
       </c>
       <c r="P459" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="Q459" t="s">
         <v>47</v>
@@ -28313,7 +28316,7 @@
     </row>
     <row r="460">
       <c r="A460" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B460" t="s">
         <v>34</v>
@@ -28334,10 +28337,10 @@
         <v>41</v>
       </c>
       <c r="H460" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="I460" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="J460" t="s">
         <v>133</v>
@@ -28346,10 +28349,10 @@
         <v>133</v>
       </c>
       <c r="L460" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M460" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N460" t="s">
         <v>47</v>
@@ -28358,7 +28361,7 @@
         <v>507</v>
       </c>
       <c r="P460" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="Q460" t="s">
         <v>47</v>
@@ -28369,7 +28372,7 @@
     </row>
     <row r="461">
       <c r="A461" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B461" t="s">
         <v>34</v>
@@ -28390,10 +28393,10 @@
         <v>41</v>
       </c>
       <c r="H461" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="I461" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="J461" t="s">
         <v>83</v>
@@ -28402,10 +28405,10 @@
         <v>119</v>
       </c>
       <c r="L461" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M461" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N461" t="s">
         <v>47</v>
@@ -28414,7 +28417,7 @@
         <v>284</v>
       </c>
       <c r="P461" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="Q461" t="s">
         <v>47</v>
@@ -28425,7 +28428,7 @@
     </row>
     <row r="462">
       <c r="A462" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B462" t="s">
         <v>34</v>
@@ -28446,10 +28449,10 @@
         <v>41</v>
       </c>
       <c r="H462" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I462" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="J462" t="s">
         <v>134</v>
@@ -28458,10 +28461,10 @@
         <v>70</v>
       </c>
       <c r="L462" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M462" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N462" t="s">
         <v>47</v>
@@ -28470,7 +28473,7 @@
         <v>155</v>
       </c>
       <c r="P462" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="Q462" t="s">
         <v>47</v>
@@ -28481,7 +28484,7 @@
     </row>
     <row r="463">
       <c r="A463" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B463" t="s">
         <v>34</v>
@@ -28502,10 +28505,10 @@
         <v>41</v>
       </c>
       <c r="H463" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I463" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="J463" t="s">
         <v>133</v>
@@ -28514,10 +28517,10 @@
         <v>133</v>
       </c>
       <c r="L463" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M463" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N463" t="s">
         <v>47</v>
@@ -28526,7 +28529,7 @@
         <v>214</v>
       </c>
       <c r="P463" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="Q463" t="s">
         <v>47</v>
@@ -28537,7 +28540,7 @@
     </row>
     <row r="464">
       <c r="A464" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B464" t="s">
         <v>34</v>
@@ -28558,10 +28561,10 @@
         <v>41</v>
       </c>
       <c r="H464" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I464" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="J464" t="s">
         <v>58</v>
@@ -28570,10 +28573,10 @@
         <v>58</v>
       </c>
       <c r="L464" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M464" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N464" t="s">
         <v>47</v>
@@ -28582,7 +28585,7 @@
         <v>259</v>
       </c>
       <c r="P464" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="Q464" t="s">
         <v>47</v>
@@ -28593,7 +28596,7 @@
     </row>
     <row r="465">
       <c r="A465" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B465" t="s">
         <v>34</v>
@@ -28614,10 +28617,10 @@
         <v>41</v>
       </c>
       <c r="H465" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I465" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="J465" t="s">
         <v>102</v>
@@ -28626,10 +28629,10 @@
         <v>102</v>
       </c>
       <c r="L465" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M465" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N465" t="s">
         <v>47</v>
@@ -28638,7 +28641,7 @@
         <v>103</v>
       </c>
       <c r="P465" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="Q465" t="s">
         <v>47</v>
@@ -28649,7 +28652,7 @@
     </row>
     <row r="466">
       <c r="A466" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B466" t="s">
         <v>34</v>
@@ -28670,10 +28673,10 @@
         <v>41</v>
       </c>
       <c r="H466" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I466" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="J466" t="s">
         <v>111</v>
@@ -28682,10 +28685,10 @@
         <v>70</v>
       </c>
       <c r="L466" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M466" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N466" t="s">
         <v>47</v>
@@ -28694,7 +28697,7 @@
         <v>289</v>
       </c>
       <c r="P466" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="Q466" t="s">
         <v>47</v>
@@ -28705,7 +28708,7 @@
     </row>
     <row r="467">
       <c r="A467" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B467" t="s">
         <v>34</v>
@@ -28726,10 +28729,10 @@
         <v>41</v>
       </c>
       <c r="H467" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I467" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="J467" t="s">
         <v>107</v>
@@ -28738,10 +28741,10 @@
         <v>107</v>
       </c>
       <c r="L467" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M467" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N467" t="s">
         <v>47</v>
@@ -28750,7 +28753,7 @@
         <v>108</v>
       </c>
       <c r="P467" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="Q467" t="s">
         <v>47</v>
@@ -28761,7 +28764,7 @@
     </row>
     <row r="468">
       <c r="A468" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B468" t="s">
         <v>34</v>
@@ -28782,10 +28785,10 @@
         <v>41</v>
       </c>
       <c r="H468" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I468" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="J468" t="s">
         <v>89</v>
@@ -28794,10 +28797,10 @@
         <v>70</v>
       </c>
       <c r="L468" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M468" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N468" t="s">
         <v>47</v>
@@ -28806,7 +28809,7 @@
         <v>164</v>
       </c>
       <c r="P468" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="Q468" t="s">
         <v>47</v>
@@ -28817,7 +28820,7 @@
     </row>
     <row r="469">
       <c r="A469" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B469" t="s">
         <v>34</v>
@@ -28838,10 +28841,10 @@
         <v>41</v>
       </c>
       <c r="H469" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I469" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="J469" t="s">
         <v>83</v>
@@ -28850,10 +28853,10 @@
         <v>70</v>
       </c>
       <c r="L469" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M469" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N469" t="s">
         <v>47</v>
@@ -28862,7 +28865,7 @@
         <v>179</v>
       </c>
       <c r="P469" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="Q469" t="s">
         <v>47</v>
@@ -28873,7 +28876,7 @@
     </row>
     <row r="470">
       <c r="A470" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B470" t="s">
         <v>34</v>
@@ -28894,10 +28897,10 @@
         <v>41</v>
       </c>
       <c r="H470" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I470" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="J470" t="s">
         <v>111</v>
@@ -28906,10 +28909,10 @@
         <v>111</v>
       </c>
       <c r="L470" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M470" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N470" t="s">
         <v>47</v>
@@ -28918,7 +28921,7 @@
         <v>112</v>
       </c>
       <c r="P470" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="Q470" t="s">
         <v>47</v>
@@ -28929,7 +28932,7 @@
     </row>
     <row r="471">
       <c r="A471" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B471" t="s">
         <v>34</v>
@@ -28950,10 +28953,10 @@
         <v>41</v>
       </c>
       <c r="H471" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I471" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="J471" t="s">
         <v>278</v>
@@ -28962,10 +28965,10 @@
         <v>70</v>
       </c>
       <c r="L471" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M471" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N471" t="s">
         <v>47</v>
@@ -28974,7 +28977,7 @@
         <v>279</v>
       </c>
       <c r="P471" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="Q471" t="s">
         <v>47</v>
@@ -28985,7 +28988,7 @@
     </row>
     <row r="472">
       <c r="A472" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B472" t="s">
         <v>34</v>
@@ -29006,10 +29009,10 @@
         <v>41</v>
       </c>
       <c r="H472" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="I472" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="J472" t="s">
         <v>119</v>
@@ -29018,10 +29021,10 @@
         <v>119</v>
       </c>
       <c r="L472" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M472" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N472" t="s">
         <v>47</v>
@@ -29030,7 +29033,7 @@
         <v>120</v>
       </c>
       <c r="P472" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="Q472" t="s">
         <v>47</v>
@@ -29041,7 +29044,7 @@
     </row>
     <row r="473">
       <c r="A473" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B473" t="s">
         <v>34</v>
@@ -29062,10 +29065,10 @@
         <v>41</v>
       </c>
       <c r="H473" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I473" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="J473" t="s">
         <v>70</v>
@@ -29074,10 +29077,10 @@
         <v>70</v>
       </c>
       <c r="L473" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M473" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N473" t="s">
         <v>47</v>
@@ -29086,7 +29089,7 @@
         <v>498</v>
       </c>
       <c r="P473" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="Q473" t="s">
         <v>47</v>
@@ -29097,7 +29100,7 @@
     </row>
     <row r="474">
       <c r="A474" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B474" t="s">
         <v>34</v>
@@ -29118,10 +29121,10 @@
         <v>41</v>
       </c>
       <c r="H474" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I474" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="J474" t="s">
         <v>83</v>
@@ -29130,10 +29133,10 @@
         <v>70</v>
       </c>
       <c r="L474" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M474" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N474" t="s">
         <v>47</v>
@@ -29142,7 +29145,7 @@
         <v>173</v>
       </c>
       <c r="P474" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="Q474" t="s">
         <v>47</v>
@@ -29153,7 +29156,7 @@
     </row>
     <row r="475">
       <c r="A475" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B475" t="s">
         <v>34</v>
@@ -29174,10 +29177,10 @@
         <v>41</v>
       </c>
       <c r="H475" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I475" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="J475" t="s">
         <v>152</v>
@@ -29186,10 +29189,10 @@
         <v>152</v>
       </c>
       <c r="L475" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M475" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N475" t="s">
         <v>47</v>
@@ -29198,7 +29201,7 @@
         <v>410</v>
       </c>
       <c r="P475" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="Q475" t="s">
         <v>47</v>
@@ -29209,7 +29212,7 @@
     </row>
     <row r="476">
       <c r="A476" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B476" t="s">
         <v>34</v>
@@ -29230,10 +29233,10 @@
         <v>41</v>
       </c>
       <c r="H476" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="I476" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="J476" t="s">
         <v>89</v>
@@ -29242,10 +29245,10 @@
         <v>70</v>
       </c>
       <c r="L476" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="M476" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="N476" t="s">
         <v>47</v>
@@ -29254,7 +29257,7 @@
         <v>490</v>
       </c>
       <c r="P476" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="Q476" t="s">
         <v>47</v>
@@ -29265,7 +29268,7 @@
     </row>
     <row r="477">
       <c r="A477" t="s" s="1">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="B477" t="s" s="1">
         <v>32</v>
@@ -29321,7 +29324,7 @@
     </row>
     <row r="478">
       <c r="A478" t="s" s="1">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="B478" t="s" s="1">
         <v>32</v>
@@ -29377,7 +29380,7 @@
     </row>
     <row r="479">
       <c r="A479" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="B479" t="s">
         <v>32</v>
@@ -29433,7 +29436,7 @@
     </row>
     <row r="480">
       <c r="A480" t="s" s="1">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="B480" t="s" s="1">
         <v>61</v>
@@ -29489,7 +29492,7 @@
     </row>
     <row r="481">
       <c r="A481" t="s" s="1">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="B481" t="s" s="1">
         <v>61</v>
@@ -29545,7 +29548,7 @@
     </row>
     <row r="482">
       <c r="A482" t="s" s="1">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="B482" t="s" s="1">
         <v>61</v>
@@ -29601,7 +29604,7 @@
     </row>
     <row r="483">
       <c r="A483" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="B483" t="s">
         <v>61</v>
@@ -29657,13 +29660,13 @@
     </row>
     <row r="484">
       <c r="A484" t="s" s="1">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="B484" t="s" s="1">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="C484" t="s" s="1">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="D484" t="s" s="1">
         <v>33</v>
@@ -29713,7 +29716,7 @@
     </row>
     <row r="485">
       <c r="A485" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="B485" t="s">
         <v>61</v>
@@ -29769,7 +29772,7 @@
     </row>
     <row r="486">
       <c r="A486" t="s" s="1">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="B486" t="s" s="1">
         <v>73</v>
@@ -29825,7 +29828,7 @@
     </row>
     <row r="487">
       <c r="A487" t="s" s="1">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="B487" t="s" s="1">
         <v>75</v>
@@ -29881,7 +29884,7 @@
     </row>
     <row r="488">
       <c r="A488" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="B488" t="s">
         <v>75</v>
@@ -29937,7 +29940,7 @@
     </row>
     <row r="489">
       <c r="A489" t="s" s="1">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="B489" t="s" s="1">
         <v>208</v>
@@ -29993,7 +29996,7 @@
     </row>
     <row r="490">
       <c r="A490" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="B490" t="s">
         <v>208</v>
@@ -30049,7 +30052,7 @@
     </row>
     <row r="491">
       <c r="A491" t="s" s="1">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="B491" t="s" s="1">
         <v>218</v>
@@ -30105,7 +30108,7 @@
     </row>
     <row r="492">
       <c r="A492" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="B492" t="s">
         <v>218</v>
@@ -30161,13 +30164,13 @@
     </row>
     <row r="493">
       <c r="A493" t="s" s="1">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="B493" t="s" s="1">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="C493" t="s" s="1">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="D493" t="s" s="1">
         <v>33</v>
@@ -30217,7 +30220,7 @@
     </row>
     <row r="494">
       <c r="A494" t="s" s="1">
-        <v>992</v>
+        <v>993</v>
       </c>
       <c r="B494" t="s" s="1">
         <v>232</v>
@@ -30273,7 +30276,7 @@
     </row>
     <row r="495">
       <c r="A495" t="s" s="1">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="B495" t="s" s="1">
         <v>234</v>
@@ -30329,7 +30332,7 @@
     </row>
     <row r="496">
       <c r="A496" t="s">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="B496" t="s">
         <v>234</v>
@@ -30385,7 +30388,7 @@
     </row>
     <row r="497">
       <c r="A497" t="s" s="1">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="B497" t="s" s="1">
         <v>354</v>
@@ -30441,7 +30444,7 @@
     </row>
     <row r="498">
       <c r="A498" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="B498" t="s">
         <v>354</v>
@@ -30497,13 +30500,13 @@
     </row>
     <row r="499">
       <c r="A499" t="s" s="1">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="B499" t="s" s="1">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="C499" t="s" s="1">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="D499" t="s" s="1">
         <v>33</v>
@@ -30553,13 +30556,13 @@
     </row>
     <row r="500">
       <c r="A500" t="s" s="1">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="B500" t="s" s="1">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="C500" t="s" s="1">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="D500" t="s" s="1">
         <v>33</v>
@@ -30609,7 +30612,7 @@
     </row>
     <row r="501">
       <c r="A501" t="s" s="1">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="B501" t="s" s="1">
         <v>478</v>
@@ -30665,7 +30668,7 @@
     </row>
     <row r="502">
       <c r="A502" t="s" s="1">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="B502" t="s" s="1">
         <v>480</v>
@@ -30721,7 +30724,7 @@
     </row>
     <row r="503">
       <c r="A503" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="B503" t="s">
         <v>480</v>
@@ -30777,7 +30780,7 @@
     </row>
     <row r="504">
       <c r="A504" t="s" s="1">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="B504" t="s" s="1">
         <v>636</v>
@@ -30833,7 +30836,7 @@
     </row>
     <row r="505">
       <c r="A505" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="B505" t="s">
         <v>636</v>
@@ -30889,7 +30892,7 @@
     </row>
     <row r="506">
       <c r="A506" t="s" s="1">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="B506" t="s" s="1">
         <v>642</v>
@@ -30945,7 +30948,7 @@
     </row>
     <row r="507">
       <c r="A507" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="B507" t="s">
         <v>644</v>
@@ -31001,7 +31004,7 @@
     </row>
     <row r="508">
       <c r="A508" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="B508" t="s">
         <v>689</v>
@@ -31057,7 +31060,7 @@
     </row>
     <row r="509">
       <c r="A509" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="B509" t="s">
         <v>702</v>
@@ -31113,7 +31116,7 @@
     </row>
     <row r="510">
       <c r="A510" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="B510" t="s">
         <v>708</v>
@@ -31169,7 +31172,7 @@
     </row>
     <row r="511">
       <c r="A511" t="s" s="1">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="B511" t="s" s="1">
         <v>732</v>
@@ -31225,7 +31228,7 @@
     </row>
     <row r="512">
       <c r="A512" t="s" s="1">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="B512" t="s" s="1">
         <v>734</v>
@@ -31281,7 +31284,7 @@
     </row>
     <row r="513">
       <c r="A513" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="B513" t="s">
         <v>736</v>
@@ -31337,7 +31340,7 @@
     </row>
     <row r="514">
       <c r="A514" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="B514" t="s">
         <v>741</v>
@@ -31393,13 +31396,13 @@
     </row>
     <row r="515">
       <c r="A515" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="B515" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="C515" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="D515" t="s">
         <v>33</v>
@@ -31449,13 +31452,13 @@
     </row>
     <row r="516">
       <c r="A516" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="B516" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="C516" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="D516" t="s">
         <v>33</v>
@@ -31505,13 +31508,13 @@
     </row>
     <row r="517">
       <c r="A517" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="B517" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="C517" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="D517" t="s">
         <v>33</v>
@@ -31561,13 +31564,13 @@
     </row>
     <row r="518">
       <c r="A518" t="s" s="1">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="B518" t="s" s="1">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="C518" t="s" s="1">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="D518" t="s" s="1">
         <v>33</v>
@@ -31617,13 +31620,13 @@
     </row>
     <row r="519">
       <c r="A519" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="B519" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="C519" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="D519" t="s">
         <v>33</v>
@@ -31673,13 +31676,13 @@
     </row>
     <row r="520">
       <c r="A520" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="B520" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="C520" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="D520" t="s">
         <v>33</v>
@@ -31729,13 +31732,13 @@
     </row>
     <row r="521">
       <c r="A521" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="B521" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="C521" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="D521" t="s">
         <v>33</v>
@@ -31785,13 +31788,13 @@
     </row>
     <row r="522">
       <c r="A522" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="B522" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="C522" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="D522" t="s">
         <v>33</v>
@@ -31841,13 +31844,13 @@
     </row>
     <row r="523">
       <c r="A523" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="B523" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="C523" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="D523" t="s">
         <v>33</v>
@@ -31897,13 +31900,13 @@
     </row>
     <row r="524">
       <c r="A524" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="B524" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="C524" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="D524" t="s">
         <v>33</v>
@@ -31953,13 +31956,13 @@
     </row>
     <row r="525">
       <c r="A525" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="B525" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="C525" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="D525" t="s">
         <v>33</v>
@@ -32009,13 +32012,13 @@
     </row>
     <row r="526">
       <c r="A526" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="B526" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="C526" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="D526" t="s">
         <v>33</v>
@@ -32065,13 +32068,13 @@
     </row>
     <row r="527">
       <c r="A527" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="B527" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="C527" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="D527" t="s">
         <v>33</v>
@@ -32121,13 +32124,13 @@
     </row>
     <row r="528">
       <c r="A528" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="B528" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="C528" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="D528" t="s">
         <v>33</v>
@@ -32177,13 +32180,13 @@
     </row>
     <row r="529">
       <c r="A529" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="B529" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="C529" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="D529" t="s">
         <v>33</v>
@@ -32233,13 +32236,13 @@
     </row>
     <row r="530">
       <c r="A530" t="s" s="1">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="B530" t="s" s="1">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="C530" t="s" s="1">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="D530" t="s" s="1">
         <v>33</v>
@@ -32289,13 +32292,13 @@
     </row>
     <row r="531">
       <c r="A531" t="s" s="1">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="B531" t="s" s="1">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="C531" t="s" s="1">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="D531" t="s" s="1">
         <v>33</v>
@@ -32345,13 +32348,13 @@
     </row>
     <row r="532">
       <c r="A532" t="s" s="1">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="B532" t="s" s="1">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="C532" t="s" s="1">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="D532" t="s" s="1">
         <v>33</v>
@@ -32401,13 +32404,13 @@
     </row>
     <row r="533">
       <c r="A533" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="B533" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="C533" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="D533" t="s">
         <v>33</v>
@@ -32457,13 +32460,13 @@
     </row>
     <row r="534">
       <c r="A534" t="s" s="1">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="B534" t="s" s="1">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="C534" t="s" s="1">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="D534" t="s" s="1">
         <v>33</v>
@@ -32513,13 +32516,13 @@
     </row>
     <row r="535">
       <c r="A535" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="B535" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="C535" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="D535" t="s">
         <v>33</v>
@@ -32569,13 +32572,13 @@
     </row>
     <row r="536">
       <c r="A536" t="s" s="1">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="B536" t="s" s="1">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="C536" t="s" s="1">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="D536" t="s" s="1">
         <v>33</v>
@@ -32625,13 +32628,13 @@
     </row>
     <row r="537">
       <c r="A537" t="s" s="1">
+        <v>1041</v>
+      </c>
+      <c r="B537" t="s" s="1">
         <v>1040</v>
       </c>
-      <c r="B537" t="s" s="1">
-        <v>1039</v>
-      </c>
       <c r="C537" t="s" s="1">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="D537" t="s" s="1">
         <v>33</v>
@@ -32681,13 +32684,13 @@
     </row>
     <row r="538">
       <c r="A538" t="s" s="1">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="B538" t="s" s="1">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="C538" t="s" s="1">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="D538" t="s" s="1">
         <v>33</v>
@@ -32737,7 +32740,7 @@
     </row>
     <row r="539">
       <c r="A539" t="s" s="1">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="B539" t="s" s="1">
         <v>73</v>
@@ -32793,13 +32796,13 @@
     </row>
     <row r="540">
       <c r="A540" t="s" s="1">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="B540" t="s" s="1">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="C540" t="s" s="1">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="D540" t="s" s="1">
         <v>33</v>
@@ -32849,7 +32852,7 @@
     </row>
     <row r="541">
       <c r="A541" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="B541" t="s">
         <v>218</v>
@@ -32905,7 +32908,7 @@
     </row>
     <row r="542">
       <c r="A542" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="B542" t="s">
         <v>232</v>
@@ -32961,7 +32964,7 @@
     </row>
     <row r="543">
       <c r="A543" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="B543" t="s">
         <v>478</v>
@@ -33017,13 +33020,13 @@
     </row>
     <row r="544">
       <c r="A544" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="B544" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="C544" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="D544" t="s">
         <v>33</v>
@@ -33073,13 +33076,13 @@
     </row>
     <row r="545">
       <c r="A545" t="s" s="1">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="B545" t="s" s="1">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="C545" t="s" s="1">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="D545" t="s" s="1">
         <v>33</v>
@@ -33129,7 +33132,7 @@
     </row>
     <row r="546">
       <c r="A546" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="B546" t="s">
         <v>732</v>
@@ -33185,13 +33188,13 @@
     </row>
     <row r="547">
       <c r="A547" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="B547" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="C547" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="D547" t="s">
         <v>33</v>
@@ -33241,7 +33244,7 @@
     </row>
     <row r="548">
       <c r="A548" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="B548" t="s">
         <v>75</v>
@@ -33297,13 +33300,13 @@
     </row>
     <row r="549">
       <c r="A549" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="B549" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="C549" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="D549" t="s">
         <v>33</v>
@@ -33353,13 +33356,13 @@
     </row>
     <row r="550">
       <c r="A550" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="B550" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="C550" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="D550" t="s">
         <v>33</v>
@@ -33409,7 +33412,7 @@
     </row>
     <row r="551">
       <c r="A551" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="B551" t="s">
         <v>234</v>
@@ -33465,7 +33468,7 @@
     </row>
     <row r="552">
       <c r="A552" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="B552" t="s">
         <v>480</v>
@@ -33521,7 +33524,7 @@
     </row>
     <row r="553">
       <c r="A553" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="B553" t="s">
         <v>734</v>
@@ -33577,13 +33580,13 @@
     </row>
     <row r="554">
       <c r="A554" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="B554" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="C554" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="D554" t="s">
         <v>33</v>
@@ -33633,7 +33636,7 @@
     </row>
     <row r="555">
       <c r="A555" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="B555" t="s">
         <v>218</v>
@@ -33689,13 +33692,13 @@
     </row>
     <row r="556">
       <c r="A556" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="B556" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="C556" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="D556" t="s">
         <v>33</v>
@@ -33745,13 +33748,13 @@
     </row>
     <row r="557">
       <c r="A557" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="B557" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="C557" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="D557" t="s">
         <v>33</v>
@@ -33801,13 +33804,13 @@
     </row>
     <row r="558">
       <c r="A558" t="s" s="1">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="B558" t="s" s="1">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="C558" t="s" s="1">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="D558" t="s" s="1">
         <v>33</v>
@@ -33857,16 +33860,16 @@
     </row>
     <row r="559">
       <c r="A559" t="s" s="1">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="B559" t="s" s="1">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="C559" t="s" s="1">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="D559" t="s" s="1">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="E559" t="s" s="1">
         <v>34</v>
@@ -33913,16 +33916,16 @@
     </row>
     <row r="560">
       <c r="A560" t="s" s="1">
+        <v>1071</v>
+      </c>
+      <c r="B560" t="s" s="1">
+        <v>1072</v>
+      </c>
+      <c r="C560" t="s" s="1">
+        <v>1072</v>
+      </c>
+      <c r="D560" t="s" s="1">
         <v>1070</v>
-      </c>
-      <c r="B560" t="s" s="1">
-        <v>1071</v>
-      </c>
-      <c r="C560" t="s" s="1">
-        <v>1071</v>
-      </c>
-      <c r="D560" t="s" s="1">
-        <v>1069</v>
       </c>
       <c r="E560" t="s" s="1">
         <v>34</v>
@@ -33969,16 +33972,16 @@
     </row>
     <row r="561">
       <c r="A561" t="s" s="1">
+        <v>1073</v>
+      </c>
+      <c r="B561" t="s" s="1">
         <v>1072</v>
       </c>
-      <c r="B561" t="s" s="1">
-        <v>1071</v>
-      </c>
       <c r="C561" t="s" s="1">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="D561" t="s" s="1">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="E561" t="s" s="1">
         <v>34</v>
@@ -34025,13 +34028,13 @@
     </row>
     <row r="562">
       <c r="A562" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="B562" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="C562" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="D562" t="s">
         <v>33</v>
@@ -34081,19 +34084,19 @@
     </row>
     <row r="563">
       <c r="A563" t="s">
+        <v>1076</v>
+      </c>
+      <c r="B563" t="s">
         <v>1075</v>
       </c>
-      <c r="B563" t="s">
-        <v>1074</v>
-      </c>
       <c r="C563" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="D563" t="s">
         <v>33</v>
       </c>
       <c r="E563" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="F563" t="s">
         <v>212</v>
@@ -34102,10 +34105,10 @@
         <v>41</v>
       </c>
       <c r="H563" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="I563" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="J563" t="s">
         <v>133</v>
@@ -34114,10 +34117,10 @@
         <v>133</v>
       </c>
       <c r="L563" t="s">
-        <v>1079</v>
+        <v>1080</v>
       </c>
       <c r="M563" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="N563" t="s">
         <v>47</v>
@@ -34126,7 +34129,7 @@
         <v>48</v>
       </c>
       <c r="P563" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="Q563" t="s">
         <v>47</v>
@@ -34137,7 +34140,7 @@
     </row>
     <row r="564">
       <c r="A564" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="B564" t="s">
         <v>34</v>
@@ -34149,7 +34152,7 @@
         <v>34</v>
       </c>
       <c r="E564" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="F564" t="s">
         <v>80</v>
@@ -34161,7 +34164,7 @@
         <v>578</v>
       </c>
       <c r="I564" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="J564" t="s">
         <v>58</v>
@@ -34170,10 +34173,10 @@
         <v>58</v>
       </c>
       <c r="L564" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="M564" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="N564" t="s">
         <v>47</v>
@@ -34182,7 +34185,7 @@
         <v>48</v>
       </c>
       <c r="P564" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="Q564" t="s">
         <v>47</v>

</xml_diff>